<commit_message>
update generated data Triggered by 9482551311a1a4a184fc73fb3e69c21e44d9fed0
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H332"/>
+  <dimension ref="A1:H333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10673,50 +10673,46 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G274" t="n">
-        <v>35.040199</v>
-      </c>
-      <c r="H274" t="n">
-        <v>-106.609001</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr"/>
+      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -10726,7 +10722,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -10740,21 +10736,21 @@
         </is>
       </c>
       <c r="G275" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H275" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -10764,7 +10760,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
@@ -10778,21 +10774,21 @@
         </is>
       </c>
       <c r="G276" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H276" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -10802,7 +10798,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -10816,21 +10812,21 @@
         </is>
       </c>
       <c r="G277" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H277" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -10840,7 +10836,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -10854,21 +10850,21 @@
         </is>
       </c>
       <c r="G278" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H278" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -10878,7 +10874,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -10892,21 +10888,21 @@
         </is>
       </c>
       <c r="G279" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H279" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10916,7 +10912,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -10930,21 +10926,21 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H280" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10954,7 +10950,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10968,21 +10964,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H281" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10992,35 +10988,35 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G282" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H282" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11030,35 +11026,35 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G283" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H283" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11068,7 +11064,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11082,21 +11078,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H284" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11106,7 +11102,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11120,21 +11116,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H285" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11144,7 +11140,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11158,21 +11154,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H286" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11182,7 +11178,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11196,21 +11192,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H287" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11220,7 +11216,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11234,21 +11230,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H288" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11258,7 +11254,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11272,21 +11268,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H289" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11296,7 +11292,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11310,21 +11306,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H290" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11334,35 +11330,35 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G291" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H291" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11372,35 +11368,35 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G292" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H292" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11410,35 +11406,35 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G293" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H293" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11448,7 +11444,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11462,21 +11458,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H294" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11486,7 +11482,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11500,21 +11496,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H295" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11524,7 +11520,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11538,21 +11534,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H296" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11562,7 +11558,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11576,21 +11572,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H297" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11600,35 +11596,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H298" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11638,35 +11634,35 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G299" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H299" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11676,7 +11672,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11690,21 +11686,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H300" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11714,7 +11710,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11728,21 +11724,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H301" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11752,35 +11748,35 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G302" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H302" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11790,35 +11786,35 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H303" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11828,7 +11824,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11842,21 +11838,21 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H304" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11866,35 +11862,35 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H305" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11904,35 +11900,35 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G306" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H306" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11942,7 +11938,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11956,21 +11952,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H307" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11980,7 +11976,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -11994,21 +11990,21 @@
         </is>
       </c>
       <c r="G308" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H308" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12018,7 +12014,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12032,21 +12028,21 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H309" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12056,7 +12052,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12070,21 +12066,21 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H310" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12094,35 +12090,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>45.322498</v>
+        <v>41.3032</v>
       </c>
       <c r="H311" t="n">
-        <v>-75.669197</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12132,35 +12128,35 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G312" t="n">
-        <v>39.871899</v>
+        <v>45.322498</v>
       </c>
       <c r="H312" t="n">
-        <v>-75.241096</v>
+        <v>-75.669197</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12170,7 +12166,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12184,21 +12180,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H313" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12208,7 +12204,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12222,21 +12218,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H314" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12246,7 +12242,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12260,21 +12256,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H315" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12284,35 +12280,35 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G316" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H316" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12322,35 +12318,35 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G317" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H317" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12360,7 +12356,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12374,21 +12370,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H318" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12398,7 +12394,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12412,21 +12408,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H319" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12436,7 +12432,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12450,21 +12446,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H320" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12474,7 +12470,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12488,21 +12484,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H321" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12512,7 +12508,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12526,21 +12522,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H322" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12550,7 +12546,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12564,21 +12560,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H323" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12588,35 +12584,35 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G324" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H324" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12626,35 +12622,35 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G325" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H325" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12664,7 +12660,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12678,21 +12674,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H326" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12702,7 +12698,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12716,21 +12712,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H327" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12740,7 +12736,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12754,21 +12750,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H328" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12778,7 +12774,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12792,21 +12788,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H329" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12816,35 +12812,35 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G330" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H330" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12854,7 +12850,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12868,47 +12864,85 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H331" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G332" t="n">
+        <v>49.193901</v>
+      </c>
+      <c r="H332" t="n">
+        <v>-123.183998</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B332" t="inlineStr">
+      <c r="B333" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C332" t="inlineStr">
+      <c r="C333" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D332" t="inlineStr">
+      <c r="D333" t="inlineStr">
         <is>
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr">
+      <c r="E333" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F332" t="inlineStr">
+      <c r="F333" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="G332" t="n">
+      <c r="G333" t="n">
         <v>49.91</v>
       </c>
-      <c r="H332" t="n">
+      <c r="H333" t="n">
         <v>-97.23989899999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 9e7cd68680540a77879c30e750829eb8c4bdc80c
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H334"/>
+  <dimension ref="A1:H335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10741,50 +10741,46 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G276" t="n">
-        <v>35.040199</v>
-      </c>
-      <c r="H276" t="n">
-        <v>-106.609001</v>
-      </c>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr"/>
+      <c r="H276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -10794,7 +10790,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -10808,21 +10804,21 @@
         </is>
       </c>
       <c r="G277" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H277" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -10832,7 +10828,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -10846,21 +10842,21 @@
         </is>
       </c>
       <c r="G278" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H278" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -10870,7 +10866,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -10884,21 +10880,21 @@
         </is>
       </c>
       <c r="G279" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H279" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10908,7 +10904,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -10922,21 +10918,21 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H280" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10946,7 +10942,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10960,21 +10956,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H281" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10984,7 +10980,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10998,21 +10994,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H282" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11022,7 +11018,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11036,21 +11032,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H283" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11060,35 +11056,35 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G284" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H284" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11098,35 +11094,35 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G285" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H285" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11136,7 +11132,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11150,21 +11146,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H286" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11174,7 +11170,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11188,21 +11184,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H287" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11212,7 +11208,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11226,21 +11222,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H288" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11250,7 +11246,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11264,21 +11260,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H289" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11288,7 +11284,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11302,21 +11298,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H290" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11326,7 +11322,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11340,21 +11336,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H291" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11364,7 +11360,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11378,21 +11374,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H292" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11402,35 +11398,35 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G293" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H293" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11440,35 +11436,35 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G294" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H294" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11478,35 +11474,35 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G295" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H295" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11516,7 +11512,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11530,21 +11526,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H296" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11554,7 +11550,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11568,21 +11564,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H297" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11592,7 +11588,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -11606,21 +11602,21 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H298" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11630,7 +11626,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11644,21 +11640,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H299" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11668,35 +11664,35 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G300" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H300" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11706,35 +11702,35 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G301" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H301" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11744,7 +11740,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11758,21 +11754,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H302" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11782,7 +11778,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11796,21 +11792,21 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H303" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11820,35 +11816,35 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G304" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H304" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11858,35 +11854,35 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H305" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11896,7 +11892,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11910,21 +11906,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H306" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11934,35 +11930,35 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H307" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11972,35 +11968,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H308" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12010,7 +12006,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12024,21 +12020,21 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H309" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12048,7 +12044,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12062,21 +12058,21 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H310" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12086,7 +12082,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12100,21 +12096,21 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H311" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12124,7 +12120,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12138,21 +12134,21 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H312" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12162,35 +12158,35 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G313" t="n">
-        <v>45.322498</v>
+        <v>41.3032</v>
       </c>
       <c r="H313" t="n">
-        <v>-75.669197</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12200,35 +12196,35 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G314" t="n">
-        <v>39.871899</v>
+        <v>45.322498</v>
       </c>
       <c r="H314" t="n">
-        <v>-75.241096</v>
+        <v>-75.669197</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12238,7 +12234,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12252,21 +12248,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H315" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12276,7 +12272,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12290,21 +12286,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H316" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12314,7 +12310,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12328,21 +12324,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H317" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12352,35 +12348,35 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G318" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H318" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12390,35 +12386,35 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G319" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H319" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12428,7 +12424,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12442,21 +12438,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H320" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12466,7 +12462,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12480,21 +12476,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H321" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12504,7 +12500,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12518,21 +12514,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H322" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12542,7 +12538,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12556,21 +12552,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H323" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12580,7 +12576,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12594,21 +12590,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H324" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12618,7 +12614,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12632,21 +12628,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H325" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12656,35 +12652,35 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G326" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H326" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12694,35 +12690,35 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G327" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H327" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12732,7 +12728,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12746,21 +12742,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H328" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12770,7 +12766,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12784,21 +12780,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H329" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12808,7 +12804,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12822,21 +12818,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H330" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12846,7 +12842,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12860,21 +12856,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H331" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12884,35 +12880,35 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G332" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H332" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12922,7 +12918,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12936,47 +12932,85 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H333" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G334" t="n">
+        <v>49.193901</v>
+      </c>
+      <c r="H334" t="n">
+        <v>-123.183998</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B334" t="inlineStr">
+      <c r="B335" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C334" t="inlineStr">
+      <c r="C335" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr">
+      <c r="D335" t="inlineStr">
         <is>
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E334" t="inlineStr">
+      <c r="E335" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F334" t="inlineStr">
+      <c r="F335" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="G334" t="n">
+      <c r="G335" t="n">
         <v>49.91</v>
       </c>
-      <c r="H334" t="n">
+      <c r="H335" t="n">
         <v>-97.23989899999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 7bd05500995bc38e3ecf0527e9f411ddb3862ef1
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H335"/>
+  <dimension ref="A1:H336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10775,50 +10775,46 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G277" t="n">
-        <v>35.040199</v>
-      </c>
-      <c r="H277" t="n">
-        <v>-106.609001</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr"/>
+      <c r="H277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -10828,7 +10824,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -10842,21 +10838,21 @@
         </is>
       </c>
       <c r="G278" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H278" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -10866,7 +10862,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -10880,21 +10876,21 @@
         </is>
       </c>
       <c r="G279" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H279" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10904,7 +10900,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -10918,21 +10914,21 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H280" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10942,7 +10938,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10956,21 +10952,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H281" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10980,7 +10976,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10994,21 +10990,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H282" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11018,7 +11014,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11032,21 +11028,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H283" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11056,7 +11052,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11070,21 +11066,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H284" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11094,35 +11090,35 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G285" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H285" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11132,35 +11128,35 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G286" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H286" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11170,7 +11166,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11184,21 +11180,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H287" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11208,7 +11204,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11222,21 +11218,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H288" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11246,7 +11242,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11260,21 +11256,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H289" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11284,7 +11280,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11298,21 +11294,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H290" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11322,7 +11318,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11336,21 +11332,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H291" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11360,7 +11356,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11374,21 +11370,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H292" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11398,7 +11394,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11412,21 +11408,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H293" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11436,35 +11432,35 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G294" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H294" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11474,35 +11470,35 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G295" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H295" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11512,35 +11508,35 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G296" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H296" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11550,7 +11546,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11564,21 +11560,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H297" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11588,7 +11584,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -11602,21 +11598,21 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H298" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11626,7 +11622,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11640,21 +11636,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H299" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11664,7 +11660,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11678,21 +11674,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H300" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11702,35 +11698,35 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G301" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H301" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11740,35 +11736,35 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G302" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H302" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11778,7 +11774,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11792,21 +11788,21 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H303" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11816,7 +11812,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11830,21 +11826,21 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H304" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11854,35 +11850,35 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H305" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11892,35 +11888,35 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G306" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H306" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11930,7 +11926,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11944,21 +11940,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H307" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11968,35 +11964,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H308" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12006,35 +12002,35 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H309" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12044,7 +12040,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12058,21 +12054,21 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H310" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12082,7 +12078,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12096,21 +12092,21 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H311" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12120,7 +12116,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12134,21 +12130,21 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H312" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12158,7 +12154,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12172,21 +12168,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H313" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12196,35 +12192,35 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G314" t="n">
-        <v>45.322498</v>
+        <v>41.3032</v>
       </c>
       <c r="H314" t="n">
-        <v>-75.669197</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12234,35 +12230,35 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G315" t="n">
-        <v>39.871899</v>
+        <v>45.322498</v>
       </c>
       <c r="H315" t="n">
-        <v>-75.241096</v>
+        <v>-75.669197</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12272,7 +12268,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12286,21 +12282,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H316" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12310,7 +12306,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12324,21 +12320,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H317" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12348,7 +12344,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12362,21 +12358,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H318" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12386,35 +12382,35 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G319" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H319" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12424,35 +12420,35 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G320" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H320" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12462,7 +12458,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12476,21 +12472,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H321" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12500,7 +12496,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12514,21 +12510,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H322" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12538,7 +12534,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12552,21 +12548,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H323" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12576,7 +12572,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12590,21 +12586,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H324" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12614,7 +12610,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12628,21 +12624,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H325" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12652,7 +12648,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12666,21 +12662,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H326" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12690,35 +12686,35 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G327" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H327" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12728,35 +12724,35 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G328" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H328" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12766,7 +12762,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12780,21 +12776,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H329" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12804,7 +12800,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12818,21 +12814,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H330" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12842,7 +12838,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12856,21 +12852,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H331" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12880,7 +12876,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12894,21 +12890,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H332" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12918,35 +12914,35 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G333" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H333" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12956,7 +12952,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -12970,47 +12966,85 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H334" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G335" t="n">
+        <v>49.193901</v>
+      </c>
+      <c r="H335" t="n">
+        <v>-123.183998</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B335" t="inlineStr">
+      <c r="B336" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C335" t="inlineStr">
+      <c r="C336" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr">
+      <c r="D336" t="inlineStr">
         <is>
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr">
+      <c r="E336" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F335" t="inlineStr">
+      <c r="F336" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="G335" t="n">
+      <c r="G336" t="n">
         <v>49.91</v>
       </c>
-      <c r="H335" t="n">
+      <c r="H336" t="n">
         <v>-97.23989899999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 1c701c8f7d77af32b5b3c140c777196b57a7b2f9
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H337"/>
+  <dimension ref="A1:H338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10843,50 +10843,46 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G279" t="n">
-        <v>35.040199</v>
-      </c>
-      <c r="H279" t="n">
-        <v>-106.609001</v>
-      </c>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr"/>
+      <c r="H279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10896,7 +10892,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -10910,21 +10906,21 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H280" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10934,7 +10930,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10948,21 +10944,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H281" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10972,7 +10968,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10986,21 +10982,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H282" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11010,7 +11006,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11024,21 +11020,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H283" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11048,7 +11044,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11062,21 +11058,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H284" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11086,7 +11082,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11100,21 +11096,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H285" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11124,7 +11120,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11138,21 +11134,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H286" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11162,35 +11158,35 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G287" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H287" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11200,35 +11196,35 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G288" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H288" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11238,7 +11234,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11252,21 +11248,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H289" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11276,7 +11272,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11290,21 +11286,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H290" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11314,7 +11310,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11328,21 +11324,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H291" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11352,7 +11348,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11366,21 +11362,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H292" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11390,7 +11386,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11404,21 +11400,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H293" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11428,7 +11424,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11442,21 +11438,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H294" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11466,7 +11462,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11480,21 +11476,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H295" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11504,35 +11500,35 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G296" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H296" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11542,35 +11538,35 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G297" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H297" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11580,35 +11576,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H298" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11618,7 +11614,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11632,21 +11628,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H299" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11656,7 +11652,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11670,21 +11666,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H300" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11694,7 +11690,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11708,21 +11704,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H301" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11732,7 +11728,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11746,21 +11742,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H302" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11770,35 +11766,35 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H303" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11808,35 +11804,35 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G304" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H304" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11846,7 +11842,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11860,21 +11856,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H305" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11884,7 +11880,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11898,21 +11894,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H306" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11922,35 +11918,35 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H307" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11960,35 +11956,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H308" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -11998,7 +11994,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12012,21 +12008,21 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H309" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12036,35 +12032,35 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H310" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12074,35 +12070,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H311" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12112,7 +12108,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12126,21 +12122,21 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H312" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12150,7 +12146,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12164,21 +12160,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H313" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12188,7 +12184,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12202,21 +12198,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H314" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12226,7 +12222,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12240,21 +12236,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H315" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12264,35 +12260,35 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G316" t="n">
-        <v>45.322498</v>
+        <v>41.3032</v>
       </c>
       <c r="H316" t="n">
-        <v>-75.669197</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12302,35 +12298,35 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G317" t="n">
-        <v>39.871899</v>
+        <v>45.322498</v>
       </c>
       <c r="H317" t="n">
-        <v>-75.241096</v>
+        <v>-75.669197</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12340,7 +12336,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12354,21 +12350,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H318" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12378,7 +12374,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12392,21 +12388,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H319" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12416,7 +12412,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12430,21 +12426,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H320" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12454,35 +12450,35 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H321" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12492,35 +12488,35 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G322" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H322" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12530,7 +12526,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12544,21 +12540,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H323" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12568,7 +12564,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12582,21 +12578,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H324" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12606,7 +12602,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12620,21 +12616,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H325" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12644,7 +12640,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12658,21 +12654,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H326" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12682,7 +12678,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12696,21 +12692,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H327" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12720,7 +12716,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12734,21 +12730,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H328" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12758,35 +12754,35 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G329" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H329" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12796,35 +12792,35 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G330" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H330" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12834,7 +12830,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12848,21 +12844,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H331" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12872,7 +12868,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12886,21 +12882,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H332" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12910,7 +12906,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12924,21 +12920,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H333" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12948,7 +12944,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -12962,21 +12958,21 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H334" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12986,35 +12982,35 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G335" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H335" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13024,7 +13020,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13038,47 +13034,85 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H336" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
+          <t>YVR</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Vancouver, BC, Canada</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G337" t="n">
+        <v>49.193901</v>
+      </c>
+      <c r="H337" t="n">
+        <v>-123.183998</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="1" t="inlineStr">
+        <is>
           <t>YWG</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B338" t="inlineStr">
         <is>
           <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C338" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D338" t="inlineStr">
         <is>
           <t>Winnipeg</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E338" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr">
+      <c r="F338" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="G337" t="n">
+      <c r="G338" t="n">
         <v>49.91</v>
       </c>
-      <c r="H337" t="n">
+      <c r="H338" t="n">
         <v>-97.23989899999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 9f0f881bb63936a0799bfc5ef80aada78dfba4b8
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H338"/>
+  <dimension ref="A1:H339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10839,50 +10839,46 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Sambalpur</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G279" t="n">
-        <v>35.040199</v>
-      </c>
-      <c r="H279" t="n">
-        <v>-106.609001</v>
-      </c>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr"/>
+      <c r="H279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10892,7 +10888,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -10906,21 +10902,21 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H280" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10930,7 +10926,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10944,21 +10940,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H281" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10968,7 +10964,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10982,21 +10978,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H282" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11006,7 +11002,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11020,21 +11016,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H283" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11044,7 +11040,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11058,21 +11054,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H284" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11082,7 +11078,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11096,21 +11092,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H285" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11120,7 +11116,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11134,21 +11130,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H286" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11158,35 +11154,35 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G287" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H287" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11196,35 +11192,35 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G288" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H288" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11234,7 +11230,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11248,21 +11244,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H289" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11272,7 +11268,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11286,21 +11282,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H290" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11310,7 +11306,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11324,21 +11320,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H291" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11348,7 +11344,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11362,21 +11358,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H292" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11386,7 +11382,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11400,21 +11396,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H293" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11424,7 +11420,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11438,21 +11434,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H294" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11462,7 +11458,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11476,21 +11472,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H295" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11500,35 +11496,35 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G296" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H296" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11538,35 +11534,35 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G297" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H297" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11576,35 +11572,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H298" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11614,7 +11610,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11628,21 +11624,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H299" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11652,7 +11648,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11666,21 +11662,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H300" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11690,7 +11686,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11704,21 +11700,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H301" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11728,7 +11724,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11742,21 +11738,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H302" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11766,35 +11762,35 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H303" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11804,35 +11800,35 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G304" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H304" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11842,7 +11838,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11856,21 +11852,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H305" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11880,7 +11876,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11894,21 +11890,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H306" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11918,35 +11914,35 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H307" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11956,35 +11952,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H308" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -11994,7 +11990,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12008,21 +12004,21 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H309" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12032,35 +12028,35 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H310" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12070,35 +12066,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H311" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12108,7 +12104,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12122,21 +12118,21 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H312" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12146,7 +12142,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12160,21 +12156,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H313" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12184,7 +12180,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12198,21 +12194,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H314" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12222,7 +12218,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12236,21 +12232,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H315" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12260,35 +12256,35 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G316" t="n">
-        <v>45.322498</v>
+        <v>41.3032</v>
       </c>
       <c r="H316" t="n">
-        <v>-75.669197</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>YOW</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Ottawa, Canada</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12298,35 +12294,35 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Ottawa</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G317" t="n">
-        <v>39.871899</v>
+        <v>45.322498</v>
       </c>
       <c r="H317" t="n">
-        <v>-75.241096</v>
+        <v>-75.669197</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12336,7 +12332,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12350,21 +12346,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H318" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12374,7 +12370,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12388,21 +12384,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H319" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12412,7 +12408,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12426,21 +12422,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H320" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12450,35 +12446,35 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H321" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12488,35 +12484,35 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G322" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H322" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12526,7 +12522,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12540,21 +12536,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H323" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12564,7 +12560,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12578,21 +12574,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H324" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12602,7 +12598,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12616,21 +12612,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H325" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12640,7 +12636,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12654,21 +12650,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H326" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12678,7 +12674,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12692,21 +12688,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H327" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12716,7 +12712,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12730,21 +12726,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H328" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12754,35 +12750,35 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G329" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H329" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12792,35 +12788,35 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G330" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H330" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12830,7 +12826,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12844,21 +12840,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H331" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12868,7 +12864,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12882,21 +12878,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H332" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12906,7 +12902,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12920,21 +12916,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H333" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12944,7 +12940,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -12958,21 +12954,21 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H334" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12982,35 +12978,35 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G335" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H335" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13020,7 +13016,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13034,21 +13030,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H336" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13058,7 +13054,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13072,43 +13068,81 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>49.91</v>
+        <v>49.193901</v>
       </c>
       <c r="H337" t="n">
-        <v>-97.23989899999999</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G338" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H338" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="1" t="inlineStr">
+        <is>
           <t>CCP</t>
         </is>
       </c>
-      <c r="B338" t="inlineStr">
+      <c r="B339" t="inlineStr">
         <is>
           <t>Concepcion, Chile</t>
         </is>
       </c>
-      <c r="C338" t="inlineStr">
+      <c r="C339" t="inlineStr">
         <is>
           <t>South America</t>
         </is>
       </c>
-      <c r="D338" t="inlineStr">
+      <c r="D339" t="inlineStr">
         <is>
           <t>Concepcion</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr"/>
-      <c r="F338" t="inlineStr">
+      <c r="E339" t="inlineStr"/>
+      <c r="F339" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="G338" t="n">
+      <c r="G339" t="n">
         <v>-36.772701</v>
       </c>
-      <c r="H338" t="n">
+      <c r="H339" t="n">
         <v>-73.063103</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by d3914d564a2d7e716154ebcc6359a2c70efe50a2
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H339"/>
+  <dimension ref="A1:H338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2663,8 +2663,12 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+      <c r="G59" t="n">
+        <v>46.223701</v>
+      </c>
+      <c r="H59" t="n">
+        <v>14.4576</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
@@ -3985,8 +3989,12 @@
           <t>NZ</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
+      <c r="G94" t="n">
+        <v>-41.327202</v>
+      </c>
+      <c r="H94" t="n">
+        <v>174.804993</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
@@ -10747,7 +10755,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -10765,8 +10773,12 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
+      <c r="G276" t="n">
+        <v>20.2444</v>
+      </c>
+      <c r="H276" t="n">
+        <v>85.817802</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
@@ -10815,7 +10827,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -10833,8 +10845,12 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="G278" t="inlineStr"/>
-      <c r="H278" t="inlineStr"/>
+      <c r="G278" t="n">
+        <v>18.5821</v>
+      </c>
+      <c r="H278" t="n">
+        <v>73.919701</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
@@ -10849,12 +10865,12 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Sambalpur</t>
+          <t>Jharsuguda</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -10867,8 +10883,12 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="G279" t="inlineStr"/>
-      <c r="H279" t="inlineStr"/>
+      <c r="G279" t="n">
+        <v>21.9135</v>
+      </c>
+      <c r="H279" t="n">
+        <v>84.0504</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
@@ -13110,40 +13130,6 @@
       </c>
       <c r="H338" t="n">
         <v>-97.23989899999999</v>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" s="1" t="inlineStr">
-        <is>
-          <t>CCP</t>
-        </is>
-      </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>Concepcion, Chile</t>
-        </is>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>South America</t>
-        </is>
-      </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>Concepcion</t>
-        </is>
-      </c>
-      <c r="E339" t="inlineStr"/>
-      <c r="F339" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="G339" t="n">
-        <v>-36.772701</v>
-      </c>
-      <c r="H339" t="n">
-        <v>-73.063103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update generated data Triggered by fe81cba4251a295145eaefff55ba63553c92f303
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Valletta, Malta</t>
+          <t>Santa Venera, Malta</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Bogota, Colombia</t>
+          <t>Bogotá, Colombia</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Cacador, Brazil</t>
+          <t>Caçador, Brazil</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Goiania, Brazil</t>
+          <t>Goiânia, Brazil</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4916,7 +4916,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Neuquen, Argentina</t>
+          <t>Neuquén, Argentina</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Timbo, Brazil</t>
+          <t>Timbó, Brazil</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Uberlandia, Brazil</t>
+          <t>Uberlândia, Brazil</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Dar es Salaam, Tanzania</t>
+          <t>Dar Es Salaam, Tanzania</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Djibouti, Djibouti</t>
+          <t>Djibouti City, Djibouti</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Chengmai, China</t>
+          <t>Haikou, China</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Chengmai</t>
+          <t>Haikou</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -8126,7 +8126,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Shijiazhuang, China</t>
+          <t>Hengshui, China</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Shijiazhuang</t>
+          <t>Hengshui</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -8346,7 +8346,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Zibo, China</t>
+          <t>Jinan, China</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Zibo</t>
+          <t>Jinan</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -8752,7 +8752,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Male, Maldives</t>
+          <t>Malé, Maldives</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Nanchang, China</t>
+          <t>Xinyu, China</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -9434,7 +9434,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Nanchang</t>
+          <t>Xinyu</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">

</xml_diff>

<commit_message>
update generated data Triggered by d99da0868901bee99fb12c5bd45ff25791b37b32
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H338"/>
+  <dimension ref="A1:H339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13132,6 +13132,40 @@
         <v>-97.23989899999999</v>
       </c>
     </row>
+    <row r="339">
+      <c r="A339" s="1" t="inlineStr">
+        <is>
+          <t>CVG</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Hebron, United States</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Hebron</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr"/>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="G339" t="n">
+        <v>39.048801</v>
+      </c>
+      <c r="H339" t="n">
+        <v>-84.667801</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update generated data Triggered by df6935ea7e01cc796e9b4c56a39aae3c07983930
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -4199,7 +4199,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>South America</t>
+          <t>Latin America &amp; the Caribbean</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4217,12 +4217,8 @@
           <t>BR</t>
         </is>
       </c>
-      <c r="G100" t="n">
-        <v>-26.830601</v>
-      </c>
-      <c r="H100" t="n">
-        <v>-49.090302</v>
-      </c>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">

</xml_diff>

<commit_message>
update generated data Triggered by e2195628cd2e7df8d41d21eb9a833c9e9d7f4c48
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H338"/>
+  <dimension ref="A1:H337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12257,12 +12257,12 @@
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YOW</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Ottawa, Canada</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12272,35 +12272,35 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Ottawa</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G316" t="n">
-        <v>45.322498</v>
+        <v>39.871899</v>
       </c>
       <c r="H316" t="n">
-        <v>-75.669197</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12310,7 +12310,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12324,21 +12324,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>39.871899</v>
+        <v>33.434299</v>
       </c>
       <c r="H317" t="n">
-        <v>-75.241096</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12362,21 +12362,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>33.434299</v>
+        <v>40.491501</v>
       </c>
       <c r="H318" t="n">
-        <v>-112.012001</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12386,7 +12386,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12400,21 +12400,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>40.491501</v>
+        <v>45.588699</v>
       </c>
       <c r="H319" t="n">
-        <v>-80.23290299999999</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12424,35 +12424,35 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G320" t="n">
-        <v>45.588699</v>
+        <v>20.6173</v>
       </c>
       <c r="H320" t="n">
-        <v>-122.598</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12462,35 +12462,35 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>20.6173</v>
+        <v>37.505199</v>
       </c>
       <c r="H321" t="n">
-        <v>-100.185997</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12500,7 +12500,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12514,21 +12514,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>37.505199</v>
+        <v>38.6954</v>
       </c>
       <c r="H322" t="n">
-        <v>-77.31970200000001</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12538,7 +12538,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12552,21 +12552,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>38.6954</v>
+        <v>40.788399</v>
       </c>
       <c r="H323" t="n">
-        <v>-121.591003</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12576,7 +12576,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12590,21 +12590,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>40.788399</v>
+        <v>29.533701</v>
       </c>
       <c r="H324" t="n">
-        <v>-111.977997</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12628,21 +12628,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>29.533701</v>
+        <v>32.733601</v>
       </c>
       <c r="H325" t="n">
-        <v>-98.469803</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12652,7 +12652,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12666,21 +12666,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>32.733601</v>
+        <v>37.618999</v>
       </c>
       <c r="H326" t="n">
-        <v>-117.190002</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12690,7 +12690,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12704,21 +12704,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>37.618999</v>
+        <v>37.362598</v>
       </c>
       <c r="H327" t="n">
-        <v>-122.375</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12728,35 +12728,35 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G328" t="n">
-        <v>37.362598</v>
+        <v>52.170799</v>
       </c>
       <c r="H328" t="n">
-        <v>-121.929001</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12766,35 +12766,35 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G329" t="n">
-        <v>52.170799</v>
+        <v>47.449001</v>
       </c>
       <c r="H329" t="n">
-        <v>-106.699997</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12804,7 +12804,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12818,21 +12818,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>47.449001</v>
+        <v>43.582001</v>
       </c>
       <c r="H330" t="n">
-        <v>-122.308998</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12842,7 +12842,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12856,21 +12856,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>43.582001</v>
+        <v>38.748699</v>
       </c>
       <c r="H331" t="n">
-        <v>-96.74189800000001</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12880,7 +12880,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12894,21 +12894,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>38.748699</v>
+        <v>30.3965</v>
       </c>
       <c r="H332" t="n">
-        <v>-90.370003</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12918,7 +12918,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12932,21 +12932,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>30.3965</v>
+        <v>27.9755</v>
       </c>
       <c r="H333" t="n">
-        <v>-84.35030399999999</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12956,35 +12956,35 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G334" t="n">
-        <v>27.9755</v>
+        <v>43.6772</v>
       </c>
       <c r="H334" t="n">
-        <v>-82.533203</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12994,7 +12994,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13008,21 +13008,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>43.6772</v>
+        <v>49.193901</v>
       </c>
       <c r="H335" t="n">
-        <v>-79.6306</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YWG</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13032,7 +13032,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Winnipeg</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13046,21 +13046,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>49.193901</v>
+        <v>49.91</v>
       </c>
       <c r="H336" t="n">
-        <v>-123.183998</v>
+        <v>-97.23989899999999</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Cincinnati, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13070,61 +13070,23 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Hebron</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G337" t="n">
-        <v>49.91</v>
+        <v>39.048801</v>
       </c>
       <c r="H337" t="n">
-        <v>-97.23989899999999</v>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" s="1" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>Cincinnati, United States</t>
-        </is>
-      </c>
-      <c r="C338" t="inlineStr">
-        <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t>Hebron</t>
-        </is>
-      </c>
-      <c r="E338" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F338" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G338" t="n">
-        <v>39.048801</v>
-      </c>
-      <c r="H338" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by e9c14c7cbefecd3353d9b7d5d8170f24b4bb16ee
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H338"/>
+  <dimension ref="A1:H337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10305,126 +10305,122 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>NQZ</t>
+          <t>KCH</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Astana, Kazakhstan</t>
+          <t>Kuching, Malaysia</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Astana</t>
+          <t>Kuching</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="G264" t="n">
-        <v>51.022202</v>
+        <v>1.4847</v>
       </c>
       <c r="H264" t="n">
-        <v>71.466904</v>
+        <v>110.347</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>KCH</t>
+          <t>AKX</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Kuching, Malaysia</t>
+          <t>Aktobe, Kazakhstan</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Kuching</t>
+          <t>Aktyubinsk</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>KZ</t>
         </is>
       </c>
       <c r="G265" t="n">
-        <v>1.4847</v>
+        <v>50.2458</v>
       </c>
       <c r="H265" t="n">
-        <v>110.347</v>
+        <v>57.206699</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>AKX</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Aktobe, Kazakhstan</t>
+          <t>Tongren, China</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Aktyubinsk</t>
+          <t>Tongren</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>KZ</t>
-        </is>
-      </c>
-      <c r="G266" t="n">
-        <v>50.2458</v>
-      </c>
-      <c r="H266" t="n">
-        <v>57.206699</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr"/>
+      <c r="H266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>HYN</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Tongren, China</t>
+          <t>Taizhou, China</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -10434,7 +10430,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Tongren</t>
+          <t>Taizhou</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
@@ -10453,46 +10449,50 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>HYN</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Taizhou, China</t>
+          <t>Bishkek, Kyrgyzstan</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Taizhou</t>
+          <t>Bishkek</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G268" t="inlineStr"/>
-      <c r="H268" t="inlineStr"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G268" t="n">
+        <v>43.061272</v>
+      </c>
+      <c r="H268" t="n">
+        <v>74.477508</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>MLG</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Bishkek, Kyrgyzstan</t>
+          <t>Malang, Indonesia</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -10502,35 +10502,35 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Bishkek</t>
+          <t>Malang-Java Island</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="G269" t="n">
-        <v>43.061272</v>
+        <v>-7.92656</v>
       </c>
       <c r="H269" t="n">
-        <v>74.477508</v>
+        <v>112.714996</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>MLG</t>
+          <t>LHE</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Malang, Indonesia</t>
+          <t>Lahore, Pakistan</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -10540,107 +10540,103 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Malang-Java Island</t>
+          <t>Lahore</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="G270" t="n">
-        <v>-7.92656</v>
+        <v>31.521601</v>
       </c>
       <c r="H270" t="n">
-        <v>112.714996</v>
+        <v>74.403603</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>LHE</t>
+          <t>CTU</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Lahore, Pakistan</t>
+          <t>Chengdu, China</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Chengdu</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="G271" t="n">
-        <v>31.521601</v>
-      </c>
-      <c r="H271" t="n">
-        <v>74.403603</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr"/>
+      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>CTU</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Chengdu, China</t>
+          <t>Agra, India</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Asia</t>
-        </is>
-      </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t>Chengdu</t>
-        </is>
-      </c>
+          <t>Asia Pacific</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr"/>
       <c r="E272" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G272" t="inlineStr"/>
-      <c r="H272" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G272" t="n">
+        <v>27.1558</v>
+      </c>
+      <c r="H272" t="n">
+        <v>77.960899</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>CJB</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Agra, India</t>
+          <t>Coimbatore, India</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -10648,7 +10644,11 @@
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr"/>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
       <c r="E273" t="inlineStr">
         <is>
           <t>India</t>
@@ -10660,165 +10660,165 @@
         </is>
       </c>
       <c r="G273" t="n">
-        <v>27.1558</v>
+        <v>11.03</v>
       </c>
       <c r="H273" t="n">
-        <v>77.960899</v>
+        <v>77.043404</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>CJB</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Coimbatore, India</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G274" t="n">
-        <v>11.03</v>
-      </c>
-      <c r="H274" t="n">
-        <v>77.043404</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr"/>
+      <c r="H274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>ACX</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Xingyi, China</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Xingyi</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G275" t="inlineStr"/>
-      <c r="H275" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G275" t="n">
+        <v>20.2444</v>
+      </c>
+      <c r="H275" t="n">
+        <v>85.817802</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>BBI</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Bhubaneswar, India</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G276" t="n">
-        <v>20.2444</v>
-      </c>
-      <c r="H276" t="n">
-        <v>85.817802</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr"/>
+      <c r="H276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>LYA</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Luoyang, China</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Luoyang</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G277" t="inlineStr"/>
-      <c r="H277" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G277" t="n">
+        <v>18.5821</v>
+      </c>
+      <c r="H277" t="n">
+        <v>73.919701</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>PNQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Pune, India</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -10828,7 +10828,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Jharsuguda</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -10842,59 +10842,59 @@
         </is>
       </c>
       <c r="G278" t="n">
-        <v>18.5821</v>
+        <v>21.9135</v>
       </c>
       <c r="H278" t="n">
-        <v>73.919701</v>
+        <v>84.0504</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>JRG</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Sambalpur, India</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>North America</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Jharsuguda</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G279" t="n">
-        <v>21.9135</v>
+        <v>35.040199</v>
       </c>
       <c r="H279" t="n">
-        <v>84.0504</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10904,7 +10904,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -10918,21 +10918,21 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>35.040199</v>
+        <v>61.1744</v>
       </c>
       <c r="H280" t="n">
-        <v>-106.609001</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10942,7 +10942,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10956,21 +10956,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>61.1744</v>
+        <v>38.9445</v>
       </c>
       <c r="H281" t="n">
-        <v>-149.996002</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10980,7 +10980,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10994,21 +10994,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>38.9445</v>
+        <v>33.6367</v>
       </c>
       <c r="H282" t="n">
-        <v>-77.455803</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11032,21 +11032,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>33.6367</v>
+        <v>30.1945</v>
       </c>
       <c r="H283" t="n">
-        <v>-84.428101</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11070,21 +11070,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>30.1945</v>
+        <v>44.8074</v>
       </c>
       <c r="H284" t="n">
-        <v>-97.669899</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11094,7 +11094,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11108,21 +11108,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>44.8074</v>
+        <v>42.3643</v>
       </c>
       <c r="H285" t="n">
-        <v>-68.828102</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11132,7 +11132,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11146,21 +11146,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>42.3643</v>
+        <v>42.940498</v>
       </c>
       <c r="H286" t="n">
-        <v>-71.00520299999999</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11170,35 +11170,35 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G287" t="n">
-        <v>42.940498</v>
+        <v>51.113899</v>
       </c>
       <c r="H287" t="n">
-        <v>-78.732201</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11208,35 +11208,35 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G288" t="n">
-        <v>51.113899</v>
+        <v>35.214001</v>
       </c>
       <c r="H288" t="n">
-        <v>-114.019997</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11246,7 +11246,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11260,21 +11260,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>35.214001</v>
+        <v>41.9786</v>
       </c>
       <c r="H289" t="n">
-        <v>-80.9431</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11284,7 +11284,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11298,21 +11298,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>41.9786</v>
+        <v>41.411701</v>
       </c>
       <c r="H290" t="n">
-        <v>-87.90479999999999</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11336,21 +11336,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>41.411701</v>
+        <v>39.998001</v>
       </c>
       <c r="H291" t="n">
-        <v>-81.8498</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11360,7 +11360,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11374,21 +11374,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>39.998001</v>
+        <v>32.896801</v>
       </c>
       <c r="H292" t="n">
-        <v>-82.891899</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11412,21 +11412,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>32.896801</v>
+        <v>39.861698</v>
       </c>
       <c r="H293" t="n">
-        <v>-97.03800200000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11436,7 +11436,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11450,21 +11450,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>39.861698</v>
+        <v>42.212399</v>
       </c>
       <c r="H294" t="n">
-        <v>-104.672997</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11474,7 +11474,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11488,21 +11488,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>42.212399</v>
+        <v>35.877602</v>
       </c>
       <c r="H295" t="n">
-        <v>-83.35340100000001</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11512,35 +11512,35 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G296" t="n">
-        <v>35.877602</v>
+        <v>20.521799</v>
       </c>
       <c r="H296" t="n">
-        <v>-78.787498</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11550,35 +11550,35 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G297" t="n">
-        <v>20.521799</v>
+        <v>44.880798</v>
       </c>
       <c r="H297" t="n">
-        <v>-103.310997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11588,35 +11588,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>44.880798</v>
+        <v>21.318701</v>
       </c>
       <c r="H298" t="n">
-        <v>-63.508598</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11640,21 +11640,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>21.318701</v>
+        <v>29.9844</v>
       </c>
       <c r="H299" t="n">
-        <v>-157.921997</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11678,21 +11678,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>29.9844</v>
+        <v>39.7173</v>
       </c>
       <c r="H300" t="n">
-        <v>-95.34139999999999</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11702,7 +11702,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11716,21 +11716,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>39.7173</v>
+        <v>30.494101</v>
       </c>
       <c r="H301" t="n">
-        <v>-86.294403</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11740,7 +11740,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11754,21 +11754,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>30.494101</v>
+        <v>39.2976</v>
       </c>
       <c r="H302" t="n">
-        <v>-81.68789700000001</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11778,35 +11778,35 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>39.2976</v>
+        <v>17.935699</v>
       </c>
       <c r="H303" t="n">
-        <v>-94.713898</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11816,35 +11816,35 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G304" t="n">
-        <v>17.935699</v>
+        <v>36.080101</v>
       </c>
       <c r="H304" t="n">
-        <v>-76.787498</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11854,7 +11854,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11868,21 +11868,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>36.080101</v>
+        <v>33.942501</v>
       </c>
       <c r="H305" t="n">
-        <v>-115.152</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11892,7 +11892,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11906,21 +11906,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>33.942501</v>
+        <v>35.0424</v>
       </c>
       <c r="H306" t="n">
-        <v>-118.407997</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11930,35 +11930,35 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>35.0424</v>
+        <v>19.4363</v>
       </c>
       <c r="H307" t="n">
-        <v>-89.97669999999999</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11968,35 +11968,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>19.4363</v>
+        <v>25.7932</v>
       </c>
       <c r="H308" t="n">
-        <v>-99.072098</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12006,7 +12006,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12020,21 +12020,21 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>25.7932</v>
+        <v>44.882</v>
       </c>
       <c r="H309" t="n">
-        <v>-80.290604</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12044,35 +12044,35 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>44.882</v>
+        <v>45.4706</v>
       </c>
       <c r="H310" t="n">
-        <v>-93.221802</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12082,35 +12082,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>45.4706</v>
+        <v>36.1245</v>
       </c>
       <c r="H311" t="n">
-        <v>-73.740799</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12120,7 +12120,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12134,21 +12134,21 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>36.1245</v>
+        <v>40.692501</v>
       </c>
       <c r="H312" t="n">
-        <v>-86.6782</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12158,7 +12158,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12172,21 +12172,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>40.692501</v>
+        <v>36.8946</v>
       </c>
       <c r="H313" t="n">
-        <v>-74.168701</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12196,7 +12196,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12210,21 +12210,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>36.8946</v>
+        <v>35.393101</v>
       </c>
       <c r="H314" t="n">
-        <v>-76.20120199999999</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12248,21 +12248,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>35.393101</v>
+        <v>41.3032</v>
       </c>
       <c r="H315" t="n">
-        <v>-97.6007</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12286,21 +12286,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>41.3032</v>
+        <v>39.871899</v>
       </c>
       <c r="H316" t="n">
-        <v>-95.894096</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12310,7 +12310,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12324,21 +12324,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>39.871899</v>
+        <v>33.434299</v>
       </c>
       <c r="H317" t="n">
-        <v>-75.241096</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12362,21 +12362,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>33.434299</v>
+        <v>40.491501</v>
       </c>
       <c r="H318" t="n">
-        <v>-112.012001</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12386,7 +12386,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12400,21 +12400,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>40.491501</v>
+        <v>45.588699</v>
       </c>
       <c r="H319" t="n">
-        <v>-80.23290299999999</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12424,35 +12424,35 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G320" t="n">
-        <v>45.588699</v>
+        <v>20.6173</v>
       </c>
       <c r="H320" t="n">
-        <v>-122.598</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12462,35 +12462,35 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>20.6173</v>
+        <v>37.505199</v>
       </c>
       <c r="H321" t="n">
-        <v>-100.185997</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12500,7 +12500,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12514,21 +12514,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>37.505199</v>
+        <v>38.6954</v>
       </c>
       <c r="H322" t="n">
-        <v>-77.31970200000001</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12538,7 +12538,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12552,21 +12552,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>38.6954</v>
+        <v>40.788399</v>
       </c>
       <c r="H323" t="n">
-        <v>-121.591003</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12576,7 +12576,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12590,21 +12590,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>40.788399</v>
+        <v>29.533701</v>
       </c>
       <c r="H324" t="n">
-        <v>-111.977997</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12628,21 +12628,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>29.533701</v>
+        <v>32.733601</v>
       </c>
       <c r="H325" t="n">
-        <v>-98.469803</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12652,7 +12652,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12666,21 +12666,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>32.733601</v>
+        <v>37.618999</v>
       </c>
       <c r="H326" t="n">
-        <v>-117.190002</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12690,7 +12690,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12704,21 +12704,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>37.618999</v>
+        <v>37.362598</v>
       </c>
       <c r="H327" t="n">
-        <v>-122.375</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12728,35 +12728,35 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G328" t="n">
-        <v>37.362598</v>
+        <v>52.170799</v>
       </c>
       <c r="H328" t="n">
-        <v>-121.929001</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12766,35 +12766,35 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G329" t="n">
-        <v>52.170799</v>
+        <v>47.449001</v>
       </c>
       <c r="H329" t="n">
-        <v>-106.699997</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12804,7 +12804,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12818,21 +12818,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>47.449001</v>
+        <v>43.582001</v>
       </c>
       <c r="H330" t="n">
-        <v>-122.308998</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12842,7 +12842,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12856,21 +12856,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>43.582001</v>
+        <v>38.748699</v>
       </c>
       <c r="H331" t="n">
-        <v>-96.74189800000001</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12880,7 +12880,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12894,21 +12894,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>38.748699</v>
+        <v>30.3965</v>
       </c>
       <c r="H332" t="n">
-        <v>-90.370003</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12918,7 +12918,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12932,21 +12932,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>30.3965</v>
+        <v>27.9755</v>
       </c>
       <c r="H333" t="n">
-        <v>-84.35030399999999</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12956,35 +12956,35 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G334" t="n">
-        <v>27.9755</v>
+        <v>43.6772</v>
       </c>
       <c r="H334" t="n">
-        <v>-82.533203</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12994,7 +12994,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13008,21 +13008,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>43.6772</v>
+        <v>49.193901</v>
       </c>
       <c r="H335" t="n">
-        <v>-79.6306</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YWG</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13032,7 +13032,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Winnipeg</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13046,21 +13046,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>49.193901</v>
+        <v>49.91</v>
       </c>
       <c r="H336" t="n">
-        <v>-123.183998</v>
+        <v>-97.23989899999999</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Cincinnati, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13070,61 +13070,23 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Hebron</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G337" t="n">
-        <v>49.91</v>
+        <v>39.048801</v>
       </c>
       <c r="H337" t="n">
-        <v>-97.23989899999999</v>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" s="1" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>Cincinnati, United States</t>
-        </is>
-      </c>
-      <c r="C338" t="inlineStr">
-        <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t>Hebron</t>
-        </is>
-      </c>
-      <c r="E338" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F338" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G338" t="n">
-        <v>39.048801</v>
-      </c>
-      <c r="H338" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 10d4c6af7aa742f37aaae72dfd2620613b677881
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -7343,12 +7343,12 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>LLW</t>
+          <t>CZL</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Lilongwe, Malawi</t>
+          <t>Constantine, Algeria</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -7358,35 +7358,35 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Lilongwe</t>
+          <t>Constantine</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Malawi</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>DZ</t>
         </is>
       </c>
       <c r="G183" t="n">
-        <v>-13.7894</v>
+        <v>36.276001</v>
       </c>
       <c r="H183" t="n">
-        <v>33.780998</v>
+        <v>6.62039</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>CZL</t>
+          <t>DLA</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Constantine, Algeria</t>
+          <t>Douala, Cameroon</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -7396,149 +7396,149 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Constantine</t>
+          <t>Douala</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>DZ</t>
+          <t>CM</t>
         </is>
       </c>
       <c r="G184" t="n">
-        <v>36.276001</v>
+        <v>4.00608</v>
       </c>
       <c r="H184" t="n">
-        <v>6.62039</v>
+        <v>9.719480000000001</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>DLA</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Douala, Cameroon</t>
+          <t>Ahmedabad, India</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Douala</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>CM</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G185" t="n">
-        <v>4.00608</v>
+        <v>23.0772</v>
       </c>
       <c r="H185" t="n">
-        <v>9.719480000000001</v>
+        <v>72.634697</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>ALA</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Ahmedabad, India</t>
+          <t>Almaty, Kazakhstan</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Almaty</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KZ</t>
         </is>
       </c>
       <c r="G186" t="n">
-        <v>23.0772</v>
+        <v>43.3521</v>
       </c>
       <c r="H186" t="n">
-        <v>72.634697</v>
+        <v>77.040497</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>ALA</t>
+          <t>BLR</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Almaty, Kazakhstan</t>
+          <t>Bangalore, India</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Almaty</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G187" t="n">
-        <v>43.3521</v>
+        <v>13.1979</v>
       </c>
       <c r="H187" t="n">
-        <v>77.040497</v>
+        <v>77.706299</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>BLR</t>
+          <t>BKK</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Bangalore, India</t>
+          <t>Bangkok, Thailand</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -7548,35 +7548,35 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bangkok</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="G188" t="n">
-        <v>13.1979</v>
+        <v>13.6811</v>
       </c>
       <c r="H188" t="n">
-        <v>77.706299</v>
+        <v>100.747002</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>BKK</t>
+          <t>BWN</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Bangkok, Thailand</t>
+          <t>Bandar Seri Begawan, Brunei</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -7586,35 +7586,35 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Bangkok</t>
+          <t>Bandar Seri Begawan</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Brunei</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>BN</t>
         </is>
       </c>
       <c r="G189" t="n">
-        <v>13.6811</v>
+        <v>4.9442</v>
       </c>
       <c r="H189" t="n">
-        <v>100.747002</v>
+        <v>114.928001</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>BWN</t>
+          <t>CEB</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Bandar Seri Begawan, Brunei</t>
+          <t>Cebu, Philippines</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -7624,35 +7624,35 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Bandar Seri Begawan</t>
+          <t>Lapu-Lapu City</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Brunei</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>BN</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="G190" t="n">
-        <v>4.9442</v>
+        <v>10.3075</v>
       </c>
       <c r="H190" t="n">
-        <v>114.928001</v>
+        <v>123.978996</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>CEB</t>
+          <t>IXC</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Cebu, Philippines</t>
+          <t>Chandigarh, India</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -7662,107 +7662,107 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Lapu-Lapu City</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G191" t="n">
-        <v>10.3075</v>
+        <v>30.6735</v>
       </c>
       <c r="H191" t="n">
-        <v>123.978996</v>
+        <v>76.788498</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>IXC</t>
+          <t>CGD</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Chandigarh, India</t>
+          <t>Changde, China</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Changde</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G192" t="n">
-        <v>30.6735</v>
-      </c>
-      <c r="H192" t="n">
-        <v>76.788498</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>CGD</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Changde, China</t>
+          <t>Chennai, India</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Changde</t>
+          <t>Chennai</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G193" t="inlineStr"/>
-      <c r="H193" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G193" t="n">
+        <v>12.990005</v>
+      </c>
+      <c r="H193" t="n">
+        <v>80.169296</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>CGP</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Chennai, India</t>
+          <t>Chittagong, Bangladesh</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -7772,35 +7772,35 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Chittagong</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>BD</t>
         </is>
       </c>
       <c r="G194" t="n">
-        <v>12.990005</v>
+        <v>22.249599</v>
       </c>
       <c r="H194" t="n">
-        <v>80.169296</v>
+        <v>91.813301</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>CGP</t>
+          <t>CMB</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Chittagong, Bangladesh</t>
+          <t>Colombo, Sri Lanka</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -7810,35 +7810,35 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Chittagong</t>
+          <t>Colombo</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>LK</t>
         </is>
       </c>
       <c r="G195" t="n">
-        <v>22.249599</v>
+        <v>7.18076</v>
       </c>
       <c r="H195" t="n">
-        <v>91.813301</v>
+        <v>79.884102</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>CMB</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Colombo, Sri Lanka</t>
+          <t>Dhaka, Bangladesh</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -7848,145 +7848,141 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Colombo</t>
+          <t>Dhaka</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>LK</t>
+          <t>BD</t>
         </is>
       </c>
       <c r="G196" t="n">
-        <v>7.18076</v>
+        <v>23.843347</v>
       </c>
       <c r="H196" t="n">
-        <v>79.884102</v>
+        <v>90.397783</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>FUO</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Dhaka, Bangladesh</t>
+          <t>Foshan, China</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>Foshan</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Bangladesh</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>BD</t>
-        </is>
-      </c>
-      <c r="G197" t="n">
-        <v>23.843347</v>
-      </c>
-      <c r="H197" t="n">
-        <v>90.397783</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>FUO</t>
+          <t>FUK</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Foshan, China</t>
+          <t>Fukuoka, Japan</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Foshan</t>
+          <t>Fukuoka</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G198" t="inlineStr"/>
-      <c r="H198" t="inlineStr"/>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="G198" t="n">
+        <v>33.585899</v>
+      </c>
+      <c r="H198" t="n">
+        <v>130.451004</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>FUK</t>
+          <t>FOC</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Fukuoka, Japan</t>
+          <t>Fuzhou, China</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Fukuoka</t>
+          <t>Fuzhou</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="G199" t="n">
-        <v>33.585899</v>
-      </c>
-      <c r="H199" t="n">
-        <v>130.451004</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>FOC</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Fuzhou, China</t>
+          <t>Guangzhou, China</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -7996,7 +7992,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Fuzhou</t>
+          <t>Guangzhou</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -8015,12 +8011,12 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>HAK</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Guangzhou, China</t>
+          <t>Haikou, China</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -8030,7 +8026,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Guangzhou</t>
+          <t>Haikou</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -8049,118 +8045,122 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>HAK</t>
+          <t>HAN</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Haikou, China</t>
+          <t>Hanoi, Vietnam</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Haikou</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G202" t="inlineStr"/>
-      <c r="H202" t="inlineStr"/>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="G202" t="n">
+        <v>21.221201</v>
+      </c>
+      <c r="H202" t="n">
+        <v>105.806999</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>HAN</t>
+          <t>SJW</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Hanoi, Vietnam</t>
+          <t>Hengshui, China</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hengshui</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>VN</t>
-        </is>
-      </c>
-      <c r="G203" t="n">
-        <v>21.221201</v>
-      </c>
-      <c r="H203" t="n">
-        <v>105.806999</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>SJW</t>
+          <t>SGN</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Hengshui, China</t>
+          <t>Ho Chi Minh City, Vietnam</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Hengshui</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G204" t="inlineStr"/>
-      <c r="H204" t="inlineStr"/>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="G204" t="n">
+        <v>10.8188</v>
+      </c>
+      <c r="H204" t="n">
+        <v>106.652</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>SGN</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City, Vietnam</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -8170,35 +8170,31 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>Vietnam</t>
-        </is>
-      </c>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr">
         <is>
-          <t>VN</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="G205" t="n">
-        <v>10.8188</v>
+        <v>22.308901</v>
       </c>
       <c r="H205" t="n">
-        <v>106.652</v>
+        <v>113.915001</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>HYD</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Hyderabad, India</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -8208,31 +8204,35 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr"/>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G206" t="n">
-        <v>22.308901</v>
+        <v>17.231318</v>
       </c>
       <c r="H206" t="n">
-        <v>113.915001</v>
+        <v>78.429855</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>HYD</t>
+          <t>ISB</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Hyderabad, India</t>
+          <t>Islamabad, Pakistan</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -8242,35 +8242,35 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Islamabad</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="G207" t="n">
-        <v>17.231318</v>
+        <v>33.616699</v>
       </c>
       <c r="H207" t="n">
-        <v>78.429855</v>
+        <v>73.099197</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>ISB</t>
+          <t>CGK</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Islamabad, Pakistan</t>
+          <t>Jakarta, Indonesia</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -8280,107 +8280,107 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Islamabad</t>
+          <t>Jakarta</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="G208" t="n">
-        <v>33.616699</v>
+        <v>-6.12557</v>
       </c>
       <c r="H208" t="n">
-        <v>73.099197</v>
+        <v>106.655998</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>CGK</t>
+          <t>TNA</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Jakarta, Indonesia</t>
+          <t>Jinan, China</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Jakarta</t>
+          <t>Jinan</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="G209" t="n">
-        <v>-6.12557</v>
-      </c>
-      <c r="H209" t="n">
-        <v>106.655998</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr"/>
+      <c r="H209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>JHB</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Jinan, China</t>
+          <t>Johor Bahru, Malaysia</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Jinan</t>
+          <t>Senai</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G210" t="inlineStr"/>
-      <c r="H210" t="inlineStr"/>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="G210" t="n">
+        <v>1.64131</v>
+      </c>
+      <c r="H210" t="n">
+        <v>103.669998</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>JHB</t>
+          <t>KNU</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Johor Bahru, Malaysia</t>
+          <t>Kanpur, India</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -8390,35 +8390,35 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Senai</t>
+          <t>Kanpur</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G211" t="n">
-        <v>1.64131</v>
+        <v>26.399462</v>
       </c>
       <c r="H211" t="n">
-        <v>103.669998</v>
+        <v>80.42695000000001</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>KNU</t>
+          <t>KHH</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Kanpur, India</t>
+          <t>Kaohsiung City</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -8428,35 +8428,31 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Kanpur</t>
-        </is>
-      </c>
-      <c r="E212" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
+          <t>Kaohsiung City</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="G212" t="n">
-        <v>26.399462</v>
+        <v>22.577101</v>
       </c>
       <c r="H212" t="n">
-        <v>80.42695000000001</v>
+        <v>120.349998</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>KHH</t>
+          <t>KHI</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Kaohsiung City</t>
+          <t>Karachi, Pakistan</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -8466,31 +8462,35 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Kaohsiung City</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr"/>
+          <t>Karachi</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
+        </is>
+      </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="G213" t="n">
-        <v>22.577101</v>
+        <v>24.9065</v>
       </c>
       <c r="H213" t="n">
-        <v>120.349998</v>
+        <v>67.160797</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>KHI</t>
+          <t>KTM</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Karachi, Pakistan</t>
+          <t>Kathmandu, Nepal</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -8500,35 +8500,35 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Karachi</t>
+          <t>Kathmandu</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>NP</t>
         </is>
       </c>
       <c r="G214" t="n">
-        <v>24.9065</v>
+        <v>27.6966</v>
       </c>
       <c r="H214" t="n">
-        <v>67.160797</v>
+        <v>85.3591</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>KTM</t>
+          <t>CCU</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Kathmandu, Nepal</t>
+          <t>Kolkata, India</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -8538,35 +8538,35 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Kathmandu</t>
+          <t>Kolkata</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>NP</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G215" t="n">
-        <v>27.6966</v>
+        <v>22.654699</v>
       </c>
       <c r="H215" t="n">
-        <v>85.3591</v>
+        <v>88.446701</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>CCU</t>
+          <t>KJA</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Kolkata, India</t>
+          <t>Krasnoyarsk, Russia</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -8576,35 +8576,35 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Krasnoyarsk</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="G216" t="n">
-        <v>22.654699</v>
+        <v>56.172901</v>
       </c>
       <c r="H216" t="n">
-        <v>88.446701</v>
+        <v>92.493301</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>KJA</t>
+          <t>KUL</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Krasnoyarsk, Russia</t>
+          <t>Kuala Lumpur, Malaysia</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -8614,107 +8614,103 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Krasnoyarsk</t>
+          <t>Kuala Lumpur</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="G217" t="n">
-        <v>56.172901</v>
+        <v>2.74558</v>
       </c>
       <c r="H217" t="n">
-        <v>92.493301</v>
+        <v>101.709999</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>KUL</t>
+          <t>PKX</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Kuala Lumpur, Malaysia</t>
+          <t>Langfang, China</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Kuala Lumpur</t>
+          <t>Langfang</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>MY</t>
-        </is>
-      </c>
-      <c r="G218" t="n">
-        <v>2.74558</v>
-      </c>
-      <c r="H218" t="n">
-        <v>101.709999</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>PKX</t>
+          <t>MFM</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Langfang, China</t>
+          <t>Macau</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>Langfang</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
+          <t>Taipa</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G219" t="inlineStr"/>
-      <c r="H219" t="inlineStr"/>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="G219" t="n">
+        <v>22.149599</v>
+      </c>
+      <c r="H219" t="n">
+        <v>113.592003</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>MFM</t>
+          <t>MLE</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Macau</t>
+          <t>Malé, Maldives</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -8724,31 +8720,35 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Taipa</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr"/>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>MV</t>
         </is>
       </c>
       <c r="G220" t="n">
-        <v>22.149599</v>
+        <v>4.19183</v>
       </c>
       <c r="H220" t="n">
-        <v>113.592003</v>
+        <v>73.529099</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>MLE</t>
+          <t>MNL</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Malé, Maldives</t>
+          <t>Manila, Philippines</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -8758,35 +8758,35 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Manila</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Maldives</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>MV</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="G221" t="n">
-        <v>4.19183</v>
+        <v>14.5086</v>
       </c>
       <c r="H221" t="n">
-        <v>73.529099</v>
+        <v>121.019997</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>MNL</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Manila, Philippines</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -8796,35 +8796,35 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Manila</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G222" t="n">
-        <v>14.5086</v>
+        <v>19.088699</v>
       </c>
       <c r="H222" t="n">
-        <v>121.019997</v>
+        <v>72.867897</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>NAG</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>Nagpur, India</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -8834,7 +8834,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Naqpur</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -8848,21 +8848,21 @@
         </is>
       </c>
       <c r="G223" t="n">
-        <v>19.088699</v>
+        <v>21.092199</v>
       </c>
       <c r="H223" t="n">
-        <v>72.867897</v>
+        <v>79.047203</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>NAG</t>
+          <t>OKA</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Nagpur, India</t>
+          <t>Naha, Japan</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -8872,35 +8872,35 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Naqpur</t>
+          <t>Naha</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G224" t="n">
-        <v>21.092199</v>
+        <v>26.195801</v>
       </c>
       <c r="H224" t="n">
-        <v>79.047203</v>
+        <v>127.646004</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>OKA</t>
+          <t>DEL</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Naha, Japan</t>
+          <t>New Delhi, India</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -8910,35 +8910,35 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Naha</t>
+          <t>New Delhi</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G225" t="n">
-        <v>26.195801</v>
+        <v>28.5665</v>
       </c>
       <c r="H225" t="n">
-        <v>127.646004</v>
+        <v>77.103104</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>DEL</t>
+          <t>KIX</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>New Delhi, India</t>
+          <t>Osaka, Japan</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -8948,35 +8948,35 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Osaka</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G226" t="n">
-        <v>28.5665</v>
+        <v>34.427299</v>
       </c>
       <c r="H226" t="n">
-        <v>77.103104</v>
+        <v>135.244003</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>KIX</t>
+          <t>PAT</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Osaka, Japan</t>
+          <t>Patna, India</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -8986,35 +8986,35 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Osaka</t>
+          <t>Patna</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G227" t="n">
-        <v>34.427299</v>
+        <v>25.591299</v>
       </c>
       <c r="H227" t="n">
-        <v>135.244003</v>
+        <v>85.087997</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>PAT</t>
+          <t>PNH</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Patna, India</t>
+          <t>Phnom Penh, Cambodia</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -9024,179 +9024,179 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Patna</t>
+          <t>Phnom Penh</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>KH</t>
         </is>
       </c>
       <c r="G228" t="n">
-        <v>25.591299</v>
+        <v>11.5466</v>
       </c>
       <c r="H228" t="n">
-        <v>85.087997</v>
+        <v>104.844002</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>PNH</t>
+          <t>TAO</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Phnom Penh, Cambodia</t>
+          <t>Qingdao, China</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Phnom Penh</t>
+          <t>Qingdao</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>KH</t>
-        </is>
-      </c>
-      <c r="G229" t="n">
-        <v>11.5466</v>
-      </c>
-      <c r="H229" t="n">
-        <v>104.844002</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr"/>
+      <c r="H229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>TAO</t>
+          <t>ICN</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Qingdao, China</t>
+          <t>Seoul, South Korea</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Qingdao</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G230" t="inlineStr"/>
-      <c r="H230" t="inlineStr"/>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>37.469101</v>
+      </c>
+      <c r="H230" t="n">
+        <v>126.450996</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>ICN</t>
+          <t>SHA</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Seoul, South Korea</t>
+          <t>Shanghai, China</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Shanghai</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="G231" t="n">
-        <v>37.469101</v>
-      </c>
-      <c r="H231" t="n">
-        <v>126.450996</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr"/>
+      <c r="H231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>SHA</t>
+          <t>SIN</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Shanghai, China</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Shanghai</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G232" t="inlineStr"/>
-      <c r="H232" t="inlineStr"/>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="G232" t="n">
+        <v>1.35019</v>
+      </c>
+      <c r="H232" t="n">
+        <v>103.994003</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>SIN</t>
+          <t>URT</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Singapore, Singapore</t>
+          <t>Surat Thani, Thailand</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -9206,35 +9206,35 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Surat Thani</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="G233" t="n">
-        <v>1.35019</v>
+        <v>9.1326</v>
       </c>
       <c r="H233" t="n">
-        <v>103.994003</v>
+        <v>99.135597</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>URT</t>
+          <t>TPE</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Surat Thani, Thailand</t>
+          <t>Taipei</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -9244,35 +9244,31 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Surat Thani</t>
-        </is>
-      </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>Thailand</t>
-        </is>
-      </c>
+          <t>Taipei</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="G234" t="n">
-        <v>9.1326</v>
+        <v>25.0777</v>
       </c>
       <c r="H234" t="n">
-        <v>99.135597</v>
+        <v>121.233002</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>TPE</t>
+          <t>NRT</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Taipei</t>
+          <t>Tokyo, Japan</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -9282,31 +9278,35 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Taipei</t>
-        </is>
-      </c>
-      <c r="E235" t="inlineStr"/>
+          <t>Tokyo</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G235" t="n">
-        <v>25.0777</v>
+        <v>35.764702</v>
       </c>
       <c r="H235" t="n">
-        <v>121.233002</v>
+        <v>140.386002</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>NRT</t>
+          <t>ULN</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
+          <t>Ulaanbaatar, Mongolia</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -9316,35 +9316,35 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Ulan Bator</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Mongolia</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="G236" t="n">
-        <v>35.764702</v>
+        <v>47.843102</v>
       </c>
       <c r="H236" t="n">
-        <v>140.386002</v>
+        <v>106.766998</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>ULN</t>
+          <t>VTE</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Ulaanbaatar, Mongolia</t>
+          <t>Vientiane, Laos</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -9354,145 +9354,145 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Ulan Bator</t>
+          <t>Vientiane</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Mongolia</t>
+          <t>Laos</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="G237" t="n">
-        <v>47.843102</v>
+        <v>17.9883</v>
       </c>
       <c r="H237" t="n">
-        <v>106.766998</v>
+        <v>102.563004</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>VTE</t>
+          <t>KHN</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Vientiane, Laos</t>
+          <t>Xinyu, China</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Vientiane</t>
+          <t>Xinyu</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Laos</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="G238" t="n">
-        <v>17.9883</v>
-      </c>
-      <c r="H238" t="n">
-        <v>102.563004</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr"/>
+      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>KHN</t>
+          <t>EVN</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Xinyu, China</t>
+          <t>Yerevan, Armenia</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Xinyu</t>
+          <t>Yerevan</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Armenia</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G239" t="inlineStr"/>
-      <c r="H239" t="inlineStr"/>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="G239" t="n">
+        <v>40.147301</v>
+      </c>
+      <c r="H239" t="n">
+        <v>44.395901</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>EVN</t>
+          <t>JOG</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Yerevan, Armenia</t>
+          <t>Yogyakarta, Indonesia</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Yerevan</t>
+          <t>Yogyakarta-Java Island</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Armenia</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="G240" t="n">
-        <v>40.147301</v>
+        <v>-7.78818</v>
       </c>
       <c r="H240" t="n">
-        <v>44.395901</v>
+        <v>110.431999</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>JOG</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Yogyakarta, Indonesia</t>
+          <t>Cagayan de Oro, Philippines</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -9502,35 +9502,35 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Yogyakarta-Java Island</t>
+          <t>Cagayan De Oro City</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="G241" t="n">
-        <v>-7.78818</v>
+        <v>8.415620000000001</v>
       </c>
       <c r="H241" t="n">
-        <v>110.431999</v>
+        <v>124.611</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>COK</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Cagayan de Oro, Philippines</t>
+          <t>Kochi, India</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -9540,35 +9540,35 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Cagayan De Oro City</t>
+          <t>Cochin</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G242" t="n">
-        <v>8.415620000000001</v>
+        <v>10.152</v>
       </c>
       <c r="H242" t="n">
-        <v>124.611</v>
+        <v>76.401901</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>COK</t>
+          <t>DPS</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Kochi, India</t>
+          <t>Denpasar, Indonesia</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -9578,35 +9578,35 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Cochin</t>
+          <t>Denpasar-Bali Island</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="G243" t="n">
-        <v>10.152</v>
+        <v>-8.74817</v>
       </c>
       <c r="H243" t="n">
-        <v>76.401901</v>
+        <v>115.167</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>DPS</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Denpasar, Indonesia</t>
+          <t>Kannur, India</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -9616,73 +9616,69 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Denpasar-Bali Island</t>
+          <t>Mattanur</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G244" t="n">
-        <v>-8.74817</v>
+        <v>11.92</v>
       </c>
       <c r="H244" t="n">
-        <v>115.167</v>
+        <v>75.55</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>CNN</t>
+          <t>SZX</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Kannur, India</t>
+          <t>Shenzhen, China</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Mattanur</t>
+          <t>Shenzhen</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G245" t="n">
-        <v>11.92</v>
-      </c>
-      <c r="H245" t="n">
-        <v>75.55</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>SZX</t>
+          <t>KWE</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Shenzhen, China</t>
+          <t>Guiyang, China</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -9692,7 +9688,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Shenzhen</t>
+          <t>Guiyang</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -9711,12 +9707,12 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>KWE</t>
+          <t>HGH</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Guiyang, China</t>
+          <t>Shaoxing, China</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -9726,7 +9722,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Guiyang</t>
+          <t>Shaoxing</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -9745,12 +9741,12 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>HGH</t>
+          <t>CZX</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Shaoxing, China</t>
+          <t>Changzhou, China</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -9760,7 +9756,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Shaoxing</t>
+          <t>Changzhou</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -9779,12 +9775,12 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>CZX</t>
+          <t>KMG</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Changzhou, China</t>
+          <t>Kunming, China</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -9794,7 +9790,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Changzhou</t>
+          <t>Kunming</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -9813,84 +9809,84 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>KMG</t>
+          <t>CNX</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Kunming, China</t>
+          <t>Chiang Mai, Thailand</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Kunming</t>
+          <t>Chiang Mai</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G250" t="inlineStr"/>
-      <c r="H250" t="inlineStr"/>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="G250" t="n">
+        <v>18.7668</v>
+      </c>
+      <c r="H250" t="n">
+        <v>98.96260100000001</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>CNX</t>
+          <t>CGO</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Chiang Mai, Thailand</t>
+          <t>Zhengzhou, China</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Chiang Mai</t>
+          <t>Zhengzhou</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>TH</t>
-        </is>
-      </c>
-      <c r="G251" t="n">
-        <v>18.7668</v>
-      </c>
-      <c r="H251" t="n">
-        <v>98.96260100000001</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr"/>
+      <c r="H251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>CGO</t>
+          <t>TYN</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Zhengzhou, China</t>
+          <t>Yangquan, China</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -9900,7 +9896,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Zhengzhou</t>
+          <t>Yangquan</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -9919,12 +9915,12 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>TYN</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Yangquan, China</t>
+          <t>Changsha, China</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -9934,7 +9930,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Yangquan</t>
+          <t>Changsha</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -9953,12 +9949,12 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>DLC</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Changsha, China</t>
+          <t>Dalian, China</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -9968,7 +9964,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Changsha</t>
+          <t>Dalian</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -9987,12 +9983,12 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>DLC</t>
+          <t>BHY</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Dalian, China</t>
+          <t>Beihai, China</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -10002,7 +9998,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Dalian</t>
+          <t>Beihai</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -10021,12 +10017,12 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>BHY</t>
+          <t>CKG</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Beihai, China</t>
+          <t>Chongqing, China</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -10036,7 +10032,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Beihai</t>
+          <t>Chongqing</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -10055,12 +10051,12 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>CKG</t>
+          <t>XFN</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Chongqing, China</t>
+          <t>Xiangyang, China</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -10070,7 +10066,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Chongqing</t>
+          <t>Xiangyang</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -10089,118 +10085,122 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>XFN</t>
+          <t>DAD</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Xiangyang, China</t>
+          <t>Da Nang, Vietnam</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Xiangyang</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G258" t="inlineStr"/>
-      <c r="H258" t="inlineStr"/>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>16.0439</v>
+      </c>
+      <c r="H258" t="n">
+        <v>108.198997</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>DAD</t>
+          <t>JXG</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Da Nang, Vietnam</t>
+          <t>Jiaxing, China</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Jiaxing</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>VN</t>
-        </is>
-      </c>
-      <c r="G259" t="n">
-        <v>16.0439</v>
-      </c>
-      <c r="H259" t="n">
-        <v>108.198997</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>JXG</t>
+          <t>CRK</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Jiaxing, China</t>
+          <t>Tarlac City, Philippines</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Jiaxing</t>
+          <t>Angeles City</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G260" t="inlineStr"/>
-      <c r="H260" t="inlineStr"/>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>15.186</v>
+      </c>
+      <c r="H260" t="n">
+        <v>120.559998</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>CRK</t>
+          <t>PBH</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Tarlac City, Philippines</t>
+          <t>Thimphu, Bhutan</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -10210,183 +10210,179 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Angeles City</t>
+          <t>Paro</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>BT</t>
         </is>
       </c>
       <c r="G261" t="n">
-        <v>15.186</v>
+        <v>27.4032</v>
       </c>
       <c r="H261" t="n">
-        <v>120.559998</v>
+        <v>89.424599</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>PBH</t>
+          <t>XIY</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Thimphu, Bhutan</t>
+          <t>Baoji, China</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Paro</t>
+          <t>Baoji</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>BT</t>
-        </is>
-      </c>
-      <c r="G262" t="n">
-        <v>27.4032</v>
-      </c>
-      <c r="H262" t="n">
-        <v>89.424599</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr"/>
+      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>XIY</t>
+          <t>KCH</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Baoji, China</t>
+          <t>Kuching, Malaysia</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Baoji</t>
+          <t>Kuching</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G263" t="inlineStr"/>
-      <c r="H263" t="inlineStr"/>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>1.4847</v>
+      </c>
+      <c r="H263" t="n">
+        <v>110.347</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>KCH</t>
+          <t>AKX</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Kuching, Malaysia</t>
+          <t>Aktobe, Kazakhstan</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Kuching</t>
+          <t>Aktyubinsk</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>KZ</t>
         </is>
       </c>
       <c r="G264" t="n">
-        <v>1.4847</v>
+        <v>50.2458</v>
       </c>
       <c r="H264" t="n">
-        <v>110.347</v>
+        <v>57.206699</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>AKX</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Aktobe, Kazakhstan</t>
+          <t>Tongren, China</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Aktyubinsk</t>
+          <t>Tongren</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>KZ</t>
-        </is>
-      </c>
-      <c r="G265" t="n">
-        <v>50.2458</v>
-      </c>
-      <c r="H265" t="n">
-        <v>57.206699</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr"/>
+      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>HYN</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Tongren, China</t>
+          <t>Taizhou, China</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -10396,7 +10392,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Tongren</t>
+          <t>Taizhou</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -10415,46 +10411,50 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>HYN</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Taizhou, China</t>
+          <t>Bishkek, Kyrgyzstan</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Taizhou</t>
+          <t>Bishkek</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G267" t="inlineStr"/>
-      <c r="H267" t="inlineStr"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>43.061272</v>
+      </c>
+      <c r="H267" t="n">
+        <v>74.477508</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>MLG</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Bishkek, Kyrgyzstan</t>
+          <t>Malang, Indonesia</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -10464,35 +10464,35 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Bishkek</t>
+          <t>Malang-Java Island</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="G268" t="n">
-        <v>43.061272</v>
+        <v>-7.92656</v>
       </c>
       <c r="H268" t="n">
-        <v>74.477508</v>
+        <v>112.714996</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>MLG</t>
+          <t>LHE</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Malang, Indonesia</t>
+          <t>Lahore, Pakistan</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -10502,107 +10502,103 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Malang-Java Island</t>
+          <t>Lahore</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="G269" t="n">
-        <v>-7.92656</v>
+        <v>31.521601</v>
       </c>
       <c r="H269" t="n">
-        <v>112.714996</v>
+        <v>74.403603</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>LHE</t>
+          <t>CTU</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Lahore, Pakistan</t>
+          <t>Chengdu, China</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Chengdu</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="G270" t="n">
-        <v>31.521601</v>
-      </c>
-      <c r="H270" t="n">
-        <v>74.403603</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr"/>
+      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>CTU</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Chengdu, China</t>
+          <t>Agra, India</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Asia</t>
-        </is>
-      </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>Chengdu</t>
-        </is>
-      </c>
+          <t>Asia Pacific</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr"/>
       <c r="E271" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G271" t="inlineStr"/>
-      <c r="H271" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G271" t="n">
+        <v>27.1558</v>
+      </c>
+      <c r="H271" t="n">
+        <v>77.960899</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>CJB</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Agra, India</t>
+          <t>Coimbatore, India</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -10610,7 +10606,11 @@
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr"/>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
       <c r="E272" t="inlineStr">
         <is>
           <t>India</t>
@@ -10622,165 +10622,165 @@
         </is>
       </c>
       <c r="G272" t="n">
-        <v>27.1558</v>
+        <v>11.03</v>
       </c>
       <c r="H272" t="n">
-        <v>77.960899</v>
+        <v>77.043404</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>CJB</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Coimbatore, India</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G273" t="n">
-        <v>11.03</v>
-      </c>
-      <c r="H273" t="n">
-        <v>77.043404</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr"/>
+      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>ACX</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Xingyi, China</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Xingyi</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G274" t="inlineStr"/>
-      <c r="H274" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G274" t="n">
+        <v>20.2444</v>
+      </c>
+      <c r="H274" t="n">
+        <v>85.817802</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>BBI</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Bhubaneswar, India</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G275" t="n">
-        <v>20.2444</v>
-      </c>
-      <c r="H275" t="n">
-        <v>85.817802</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr"/>
+      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>LYA</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Luoyang, China</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Luoyang</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G276" t="n">
+        <v>18.5821</v>
+      </c>
+      <c r="H276" t="n">
+        <v>73.919701</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>PNQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Pune, India</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -10790,7 +10790,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Jharsuguda</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -10804,49 +10804,45 @@
         </is>
       </c>
       <c r="G277" t="n">
-        <v>18.5821</v>
+        <v>21.9135</v>
       </c>
       <c r="H277" t="n">
-        <v>73.919701</v>
+        <v>84.0504</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>JRG</t>
+          <t>AVA</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Sambalpur, India</t>
+          <t>Anshun, China</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Jharsuguda</t>
+          <t>Anshun</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G278" t="n">
-        <v>21.9135</v>
-      </c>
-      <c r="H278" t="n">
-        <v>84.0504</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr"/>
+      <c r="H278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">

</xml_diff>

<commit_message>
update generated data Triggered by e6454c899c55700c429b4996a888b5d60747850b
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H337"/>
+  <dimension ref="A1:H338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10847,50 +10847,50 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>NQZ</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Astana, Kazakhstan</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Astana</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KZ</t>
         </is>
       </c>
       <c r="G279" t="n">
-        <v>35.040199</v>
+        <v>51.022202</v>
       </c>
       <c r="H279" t="n">
-        <v>-106.609001</v>
+        <v>71.466904</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10900,7 +10900,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -10914,21 +10914,21 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H280" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10938,7 +10938,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10952,21 +10952,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H281" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10976,7 +10976,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10990,21 +10990,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H282" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11028,21 +11028,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H283" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11052,7 +11052,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11066,21 +11066,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H284" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11090,7 +11090,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11104,21 +11104,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H285" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11128,7 +11128,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11142,21 +11142,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H286" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11166,35 +11166,35 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G287" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H287" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11204,35 +11204,35 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G288" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H288" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11256,21 +11256,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H289" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11294,21 +11294,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H290" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11318,7 +11318,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11332,21 +11332,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H291" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11370,21 +11370,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H292" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11408,21 +11408,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H293" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11432,7 +11432,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11446,21 +11446,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H294" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11470,7 +11470,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11484,21 +11484,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H295" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11508,35 +11508,35 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G296" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H296" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11546,35 +11546,35 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G297" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H297" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11584,35 +11584,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H298" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11622,7 +11622,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11636,21 +11636,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H299" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11660,7 +11660,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11674,21 +11674,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H300" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11698,7 +11698,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11712,21 +11712,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H301" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11736,7 +11736,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11750,21 +11750,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H302" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11774,35 +11774,35 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H303" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11812,35 +11812,35 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G304" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H304" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11850,7 +11850,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11864,21 +11864,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H305" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11902,21 +11902,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H306" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11926,35 +11926,35 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H307" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11964,35 +11964,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H308" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12002,7 +12002,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12016,21 +12016,21 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H309" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12040,35 +12040,35 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H310" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12078,35 +12078,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H311" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12116,7 +12116,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12130,21 +12130,21 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H312" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12154,7 +12154,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12168,21 +12168,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H313" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12192,7 +12192,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12206,21 +12206,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H314" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12244,21 +12244,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H315" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12268,7 +12268,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12282,21 +12282,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>39.871899</v>
+        <v>41.3032</v>
       </c>
       <c r="H316" t="n">
-        <v>-75.241096</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12306,7 +12306,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12320,21 +12320,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H317" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12344,7 +12344,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12358,21 +12358,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H318" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12382,7 +12382,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12396,21 +12396,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H319" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12420,35 +12420,35 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G320" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H320" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12458,35 +12458,35 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H321" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12496,7 +12496,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12510,21 +12510,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H322" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12534,7 +12534,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12548,21 +12548,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H323" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12586,21 +12586,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H324" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12610,7 +12610,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12624,21 +12624,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H325" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12648,7 +12648,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12662,21 +12662,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H326" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12686,7 +12686,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12700,21 +12700,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H327" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12724,35 +12724,35 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G328" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H328" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12762,35 +12762,35 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G329" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H329" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12800,7 +12800,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12814,21 +12814,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H330" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12838,7 +12838,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12852,21 +12852,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H331" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12876,7 +12876,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12890,21 +12890,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H332" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12914,7 +12914,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12928,21 +12928,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H333" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12952,35 +12952,35 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G334" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H334" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12990,7 +12990,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13004,21 +13004,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H335" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13028,7 +13028,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13042,47 +13042,85 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>49.91</v>
+        <v>49.193901</v>
       </c>
       <c r="H336" t="n">
-        <v>-97.23989899999999</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G337" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H337" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B338" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C338" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D338" t="inlineStr">
         <is>
           <t>Hebron</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E338" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F337" t="inlineStr">
+      <c r="F338" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G337" t="n">
+      <c r="G338" t="n">
         <v>39.048801</v>
       </c>
-      <c r="H337" t="n">
+      <c r="H338" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 326a63d42efcec79998f9de6df5e03a15106135d
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H338"/>
+  <dimension ref="A1:H339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10885,50 +10885,50 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>BDQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Jamnagar, India</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Vadodara</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G280" t="n">
-        <v>35.040199</v>
+        <v>22.336201</v>
       </c>
       <c r="H280" t="n">
-        <v>-106.609001</v>
+        <v>73.226303</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -10938,7 +10938,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -10952,21 +10952,21 @@
         </is>
       </c>
       <c r="G281" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H281" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10976,7 +10976,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10990,21 +10990,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H282" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11028,21 +11028,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H283" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11052,7 +11052,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11066,21 +11066,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H284" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11090,7 +11090,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11104,21 +11104,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H285" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11128,7 +11128,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11142,21 +11142,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H286" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11180,21 +11180,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H287" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11204,35 +11204,35 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G288" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H288" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11242,35 +11242,35 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G289" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H289" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11294,21 +11294,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H290" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11318,7 +11318,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11332,21 +11332,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H291" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11370,21 +11370,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H292" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11408,21 +11408,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H293" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11432,7 +11432,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11446,21 +11446,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H294" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11470,7 +11470,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11484,21 +11484,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H295" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11508,7 +11508,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11522,21 +11522,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H296" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11546,35 +11546,35 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G297" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H297" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11584,35 +11584,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H298" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11622,35 +11622,35 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G299" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H299" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11660,7 +11660,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11674,21 +11674,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H300" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11698,7 +11698,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11712,21 +11712,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H301" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11736,7 +11736,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11750,21 +11750,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H302" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11774,7 +11774,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11788,21 +11788,21 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H303" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11812,35 +11812,35 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G304" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H304" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11850,35 +11850,35 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H305" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11888,7 +11888,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11902,21 +11902,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H306" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11926,7 +11926,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11940,21 +11940,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H307" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11964,35 +11964,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H308" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12002,35 +12002,35 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H309" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12040,7 +12040,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12054,21 +12054,21 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H310" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12078,35 +12078,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H311" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12116,35 +12116,35 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G312" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H312" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12154,7 +12154,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12168,21 +12168,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H313" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12192,7 +12192,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12206,21 +12206,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H314" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12244,21 +12244,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H315" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12268,7 +12268,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12282,21 +12282,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H316" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12306,7 +12306,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12320,21 +12320,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>39.871899</v>
+        <v>41.3032</v>
       </c>
       <c r="H317" t="n">
-        <v>-75.241096</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12344,7 +12344,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12358,21 +12358,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H318" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12382,7 +12382,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12396,21 +12396,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H319" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12420,7 +12420,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12434,21 +12434,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H320" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12458,35 +12458,35 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G321" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H321" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12496,35 +12496,35 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G322" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H322" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12534,7 +12534,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12548,21 +12548,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H323" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12586,21 +12586,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H324" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12610,7 +12610,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12624,21 +12624,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H325" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12648,7 +12648,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12662,21 +12662,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H326" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12686,7 +12686,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12700,21 +12700,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H327" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12724,7 +12724,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12738,21 +12738,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H328" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12762,35 +12762,35 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G329" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H329" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12800,35 +12800,35 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G330" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H330" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12838,7 +12838,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12852,21 +12852,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H331" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12876,7 +12876,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12890,21 +12890,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H332" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12914,7 +12914,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12928,21 +12928,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H333" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12952,7 +12952,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -12966,21 +12966,21 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H334" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12990,35 +12990,35 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G335" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H335" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13028,7 +13028,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13042,21 +13042,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H336" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13066,7 +13066,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13080,47 +13080,85 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>49.91</v>
+        <v>49.193901</v>
       </c>
       <c r="H337" t="n">
-        <v>-97.23989899999999</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G338" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H338" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B338" t="inlineStr">
+      <c r="B339" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C338" t="inlineStr">
+      <c r="C339" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D338" t="inlineStr">
+      <c r="D339" t="inlineStr">
         <is>
           <t>Hebron</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr">
+      <c r="E339" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F338" t="inlineStr">
+      <c r="F339" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G338" t="n">
+      <c r="G339" t="n">
         <v>39.048801</v>
       </c>
-      <c r="H338" t="n">
+      <c r="H339" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 3ce205b1a310a26794db8dfb6a3b8faa4eb35523
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H340"/>
+  <dimension ref="A1:H339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10021,12 +10021,12 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>BHY</t>
+          <t>CKG</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Beihai, China</t>
+          <t>Chongqing, China</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -10036,7 +10036,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Beihai</t>
+          <t>Chongqing</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -10055,12 +10055,12 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>CKG</t>
+          <t>XFN</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Chongqing, China</t>
+          <t>Xiangyang, China</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -10070,7 +10070,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Chongqing</t>
+          <t>Xiangyang</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -10089,118 +10089,122 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>XFN</t>
+          <t>DAD</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Xiangyang, China</t>
+          <t>Da Nang, Vietnam</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Xiangyang</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G258" t="inlineStr"/>
-      <c r="H258" t="inlineStr"/>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>16.0439</v>
+      </c>
+      <c r="H258" t="n">
+        <v>108.198997</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>DAD</t>
+          <t>JXG</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Da Nang, Vietnam</t>
+          <t>Jiaxing, China</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Jiaxing</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>VN</t>
-        </is>
-      </c>
-      <c r="G259" t="n">
-        <v>16.0439</v>
-      </c>
-      <c r="H259" t="n">
-        <v>108.198997</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>JXG</t>
+          <t>CRK</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Jiaxing, China</t>
+          <t>Tarlac City, Philippines</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Jiaxing</t>
+          <t>Angeles City</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G260" t="inlineStr"/>
-      <c r="H260" t="inlineStr"/>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>15.186</v>
+      </c>
+      <c r="H260" t="n">
+        <v>120.559998</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>CRK</t>
+          <t>PBH</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Tarlac City, Philippines</t>
+          <t>Thimphu, Bhutan</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -10210,183 +10214,179 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Angeles City</t>
+          <t>Paro</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>BT</t>
         </is>
       </c>
       <c r="G261" t="n">
-        <v>15.186</v>
+        <v>27.4032</v>
       </c>
       <c r="H261" t="n">
-        <v>120.559998</v>
+        <v>89.424599</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>PBH</t>
+          <t>XIY</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Thimphu, Bhutan</t>
+          <t>Baoji, China</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Paro</t>
+          <t>Baoji</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>BT</t>
-        </is>
-      </c>
-      <c r="G262" t="n">
-        <v>27.4032</v>
-      </c>
-      <c r="H262" t="n">
-        <v>89.424599</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr"/>
+      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>XIY</t>
+          <t>KCH</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Baoji, China</t>
+          <t>Kuching, Malaysia</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Baoji</t>
+          <t>Kuching</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G263" t="inlineStr"/>
-      <c r="H263" t="inlineStr"/>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>1.4847</v>
+      </c>
+      <c r="H263" t="n">
+        <v>110.347</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>KCH</t>
+          <t>AKX</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Kuching, Malaysia</t>
+          <t>Aktobe, Kazakhstan</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Kuching</t>
+          <t>Aktyubinsk</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>KZ</t>
         </is>
       </c>
       <c r="G264" t="n">
-        <v>1.4847</v>
+        <v>50.2458</v>
       </c>
       <c r="H264" t="n">
-        <v>110.347</v>
+        <v>57.206699</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>AKX</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Aktobe, Kazakhstan</t>
+          <t>Tongren, China</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Aktyubinsk</t>
+          <t>Tongren</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>KZ</t>
-        </is>
-      </c>
-      <c r="G265" t="n">
-        <v>50.2458</v>
-      </c>
-      <c r="H265" t="n">
-        <v>57.206699</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr"/>
+      <c r="H265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>HYN</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Tongren, China</t>
+          <t>Taizhou, China</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -10396,7 +10396,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Tongren</t>
+          <t>Taizhou</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -10415,46 +10415,50 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>HYN</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Taizhou, China</t>
+          <t>Bishkek, Kyrgyzstan</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Taizhou</t>
+          <t>Bishkek</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G267" t="inlineStr"/>
-      <c r="H267" t="inlineStr"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>43.061272</v>
+      </c>
+      <c r="H267" t="n">
+        <v>74.477508</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>MLG</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Bishkek, Kyrgyzstan</t>
+          <t>Malang, Indonesia</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -10464,35 +10468,35 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Bishkek</t>
+          <t>Malang-Java Island</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="G268" t="n">
-        <v>43.061272</v>
+        <v>-7.92656</v>
       </c>
       <c r="H268" t="n">
-        <v>74.477508</v>
+        <v>112.714996</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>MLG</t>
+          <t>LHE</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Malang, Indonesia</t>
+          <t>Lahore, Pakistan</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -10502,107 +10506,103 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Malang-Java Island</t>
+          <t>Lahore</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="G269" t="n">
-        <v>-7.92656</v>
+        <v>31.521601</v>
       </c>
       <c r="H269" t="n">
-        <v>112.714996</v>
+        <v>74.403603</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>LHE</t>
+          <t>CTU</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Lahore, Pakistan</t>
+          <t>Chengdu, China</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Lahore</t>
+          <t>Chengdu</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="G270" t="n">
-        <v>31.521601</v>
-      </c>
-      <c r="H270" t="n">
-        <v>74.403603</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr"/>
+      <c r="H270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>CTU</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Chengdu, China</t>
+          <t>Agra, India</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Asia</t>
-        </is>
-      </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>Chengdu</t>
-        </is>
-      </c>
+          <t>Asia Pacific</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr"/>
       <c r="E271" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G271" t="inlineStr"/>
-      <c r="H271" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G271" t="n">
+        <v>27.1558</v>
+      </c>
+      <c r="H271" t="n">
+        <v>77.960899</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>CJB</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Agra, India</t>
+          <t>Coimbatore, India</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -10610,7 +10610,11 @@
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr"/>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
       <c r="E272" t="inlineStr">
         <is>
           <t>India</t>
@@ -10622,165 +10626,165 @@
         </is>
       </c>
       <c r="G272" t="n">
-        <v>27.1558</v>
+        <v>11.03</v>
       </c>
       <c r="H272" t="n">
-        <v>77.960899</v>
+        <v>77.043404</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>CJB</t>
+          <t>ACX</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Coimbatore, India</t>
+          <t>Xingyi, China</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Xingyi</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G273" t="n">
-        <v>11.03</v>
-      </c>
-      <c r="H273" t="n">
-        <v>77.043404</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr"/>
+      <c r="H273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>ACX</t>
+          <t>BBI</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Xingyi, China</t>
+          <t>Bhubaneswar, India</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Xingyi</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G274" t="inlineStr"/>
-      <c r="H274" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G274" t="n">
+        <v>20.2444</v>
+      </c>
+      <c r="H274" t="n">
+        <v>85.817802</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>BBI</t>
+          <t>LYA</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Bhubaneswar, India</t>
+          <t>Luoyang, China</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Luoyang</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G275" t="n">
-        <v>20.2444</v>
-      </c>
-      <c r="H275" t="n">
-        <v>85.817802</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr"/>
+      <c r="H275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>LYA</t>
+          <t>PNQ</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Luoyang, China</t>
+          <t>Pune, India</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Luoyang</t>
+          <t>Pune</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G276" t="n">
+        <v>18.5821</v>
+      </c>
+      <c r="H276" t="n">
+        <v>73.919701</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>PNQ</t>
+          <t>JRG</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Pune, India</t>
+          <t>Sambalpur, India</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -10790,7 +10794,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Jharsuguda</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -10804,93 +10808,93 @@
         </is>
       </c>
       <c r="G277" t="n">
-        <v>18.5821</v>
+        <v>21.9135</v>
       </c>
       <c r="H277" t="n">
-        <v>73.919701</v>
+        <v>84.0504</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>JRG</t>
+          <t>AVA</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Sambalpur, India</t>
+          <t>Anshun, China</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Jharsuguda</t>
+          <t>Anshun</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="G278" t="n">
-        <v>21.9135</v>
-      </c>
-      <c r="H278" t="n">
-        <v>84.0504</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr"/>
+      <c r="H278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>AVA</t>
+          <t>NQZ</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Anshun, China</t>
+          <t>Astana, Kazakhstan</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Anshun</t>
+          <t>Astana</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G279" t="inlineStr"/>
-      <c r="H279" t="inlineStr"/>
+          <t>KZ</t>
+        </is>
+      </c>
+      <c r="G279" t="n">
+        <v>51.022202</v>
+      </c>
+      <c r="H279" t="n">
+        <v>71.466904</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>NQZ</t>
+          <t>BDQ</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Astana, Kazakhstan</t>
+          <t>Jamnagar, India</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -10900,73 +10904,73 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Astana</t>
+          <t>Vadodara</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>KZ</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G280" t="n">
-        <v>51.022202</v>
+        <v>22.336201</v>
       </c>
       <c r="H280" t="n">
-        <v>71.466904</v>
+        <v>73.226303</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>BDQ</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Jamnagar, India</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Asia Pacific</t>
+          <t>North America</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Vadodara</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G281" t="n">
-        <v>22.336201</v>
+        <v>35.040199</v>
       </c>
       <c r="H281" t="n">
-        <v>73.226303</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10976,7 +10980,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10990,21 +10994,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>35.040199</v>
+        <v>61.1744</v>
       </c>
       <c r="H282" t="n">
-        <v>-106.609001</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11014,7 +11018,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11028,21 +11032,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>61.1744</v>
+        <v>38.9445</v>
       </c>
       <c r="H283" t="n">
-        <v>-149.996002</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11052,7 +11056,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11066,21 +11070,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>38.9445</v>
+        <v>33.6367</v>
       </c>
       <c r="H284" t="n">
-        <v>-77.455803</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11090,7 +11094,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11104,21 +11108,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>33.6367</v>
+        <v>30.1945</v>
       </c>
       <c r="H285" t="n">
-        <v>-84.428101</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11128,7 +11132,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11142,21 +11146,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>30.1945</v>
+        <v>44.8074</v>
       </c>
       <c r="H286" t="n">
-        <v>-97.669899</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11166,7 +11170,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11180,21 +11184,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>44.8074</v>
+        <v>42.3643</v>
       </c>
       <c r="H287" t="n">
-        <v>-68.828102</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11204,7 +11208,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11218,21 +11222,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>42.3643</v>
+        <v>42.940498</v>
       </c>
       <c r="H288" t="n">
-        <v>-71.00520299999999</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11242,35 +11246,35 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G289" t="n">
-        <v>42.940498</v>
+        <v>51.113899</v>
       </c>
       <c r="H289" t="n">
-        <v>-78.732201</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11280,35 +11284,35 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G290" t="n">
-        <v>51.113899</v>
+        <v>35.214001</v>
       </c>
       <c r="H290" t="n">
-        <v>-114.019997</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11318,7 +11322,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11332,21 +11336,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>35.214001</v>
+        <v>41.9786</v>
       </c>
       <c r="H291" t="n">
-        <v>-80.9431</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11356,7 +11360,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11370,21 +11374,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>41.9786</v>
+        <v>41.411701</v>
       </c>
       <c r="H292" t="n">
-        <v>-87.90479999999999</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11394,7 +11398,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11408,21 +11412,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>41.411701</v>
+        <v>39.998001</v>
       </c>
       <c r="H293" t="n">
-        <v>-81.8498</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11432,7 +11436,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11446,21 +11450,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>39.998001</v>
+        <v>32.896801</v>
       </c>
       <c r="H294" t="n">
-        <v>-82.891899</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11470,7 +11474,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11484,21 +11488,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>32.896801</v>
+        <v>39.861698</v>
       </c>
       <c r="H295" t="n">
-        <v>-97.03800200000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11508,7 +11512,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11522,21 +11526,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>39.861698</v>
+        <v>42.212399</v>
       </c>
       <c r="H296" t="n">
-        <v>-104.672997</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11546,7 +11550,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11560,21 +11564,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>42.212399</v>
+        <v>35.877602</v>
       </c>
       <c r="H297" t="n">
-        <v>-83.35340100000001</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11584,35 +11588,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>35.877602</v>
+        <v>20.521799</v>
       </c>
       <c r="H298" t="n">
-        <v>-78.787498</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11622,35 +11626,35 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G299" t="n">
-        <v>20.521799</v>
+        <v>44.880798</v>
       </c>
       <c r="H299" t="n">
-        <v>-103.310997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11660,35 +11664,35 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G300" t="n">
-        <v>44.880798</v>
+        <v>21.318701</v>
       </c>
       <c r="H300" t="n">
-        <v>-63.508598</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11698,7 +11702,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11712,21 +11716,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>21.318701</v>
+        <v>29.9844</v>
       </c>
       <c r="H301" t="n">
-        <v>-157.921997</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11736,7 +11740,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11750,21 +11754,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>29.9844</v>
+        <v>39.7173</v>
       </c>
       <c r="H302" t="n">
-        <v>-95.34139999999999</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11774,7 +11778,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11788,21 +11792,21 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>39.7173</v>
+        <v>30.494101</v>
       </c>
       <c r="H303" t="n">
-        <v>-86.294403</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11812,7 +11816,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11826,21 +11830,21 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>30.494101</v>
+        <v>39.2976</v>
       </c>
       <c r="H304" t="n">
-        <v>-81.68789700000001</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11850,35 +11854,35 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>39.2976</v>
+        <v>17.935699</v>
       </c>
       <c r="H305" t="n">
-        <v>-94.713898</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11888,35 +11892,35 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G306" t="n">
-        <v>17.935699</v>
+        <v>36.080101</v>
       </c>
       <c r="H306" t="n">
-        <v>-76.787498</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11926,7 +11930,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11940,21 +11944,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>36.080101</v>
+        <v>33.942501</v>
       </c>
       <c r="H307" t="n">
-        <v>-115.152</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11964,7 +11968,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -11978,21 +11982,21 @@
         </is>
       </c>
       <c r="G308" t="n">
-        <v>33.942501</v>
+        <v>35.0424</v>
       </c>
       <c r="H308" t="n">
-        <v>-118.407997</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12002,35 +12006,35 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>35.0424</v>
+        <v>19.4363</v>
       </c>
       <c r="H309" t="n">
-        <v>-89.97669999999999</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12040,35 +12044,35 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>19.4363</v>
+        <v>25.7932</v>
       </c>
       <c r="H310" t="n">
-        <v>-99.072098</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12078,7 +12082,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12092,21 +12096,21 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>25.7932</v>
+        <v>44.882</v>
       </c>
       <c r="H311" t="n">
-        <v>-80.290604</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12116,35 +12120,35 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G312" t="n">
-        <v>44.882</v>
+        <v>45.4706</v>
       </c>
       <c r="H312" t="n">
-        <v>-93.221802</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12154,35 +12158,35 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G313" t="n">
-        <v>45.4706</v>
+        <v>36.1245</v>
       </c>
       <c r="H313" t="n">
-        <v>-73.740799</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12192,7 +12196,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12206,21 +12210,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>36.1245</v>
+        <v>40.692501</v>
       </c>
       <c r="H314" t="n">
-        <v>-86.6782</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12230,7 +12234,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12244,21 +12248,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>40.692501</v>
+        <v>36.8946</v>
       </c>
       <c r="H315" t="n">
-        <v>-74.168701</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12268,7 +12272,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12282,21 +12286,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>36.8946</v>
+        <v>35.393101</v>
       </c>
       <c r="H316" t="n">
-        <v>-76.20120199999999</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12306,7 +12310,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12320,21 +12324,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>35.393101</v>
+        <v>41.3032</v>
       </c>
       <c r="H317" t="n">
-        <v>-97.6007</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12344,7 +12348,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12358,21 +12362,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>41.3032</v>
+        <v>39.871899</v>
       </c>
       <c r="H318" t="n">
-        <v>-95.894096</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12382,7 +12386,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12396,21 +12400,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>39.871899</v>
+        <v>33.434299</v>
       </c>
       <c r="H319" t="n">
-        <v>-75.241096</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12420,7 +12424,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12434,21 +12438,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>33.434299</v>
+        <v>40.491501</v>
       </c>
       <c r="H320" t="n">
-        <v>-112.012001</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12458,7 +12462,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12472,21 +12476,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>40.491501</v>
+        <v>45.588699</v>
       </c>
       <c r="H321" t="n">
-        <v>-80.23290299999999</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12496,35 +12500,35 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G322" t="n">
-        <v>45.588699</v>
+        <v>20.6173</v>
       </c>
       <c r="H322" t="n">
-        <v>-122.598</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12534,35 +12538,35 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G323" t="n">
-        <v>20.6173</v>
+        <v>37.505199</v>
       </c>
       <c r="H323" t="n">
-        <v>-100.185997</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12572,7 +12576,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12586,21 +12590,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>37.505199</v>
+        <v>38.6954</v>
       </c>
       <c r="H324" t="n">
-        <v>-77.31970200000001</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12610,7 +12614,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12624,21 +12628,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>38.6954</v>
+        <v>40.788399</v>
       </c>
       <c r="H325" t="n">
-        <v>-121.591003</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12648,7 +12652,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12662,21 +12666,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>40.788399</v>
+        <v>29.533701</v>
       </c>
       <c r="H326" t="n">
-        <v>-111.977997</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12686,7 +12690,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12700,21 +12704,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>29.533701</v>
+        <v>32.733601</v>
       </c>
       <c r="H327" t="n">
-        <v>-98.469803</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12724,7 +12728,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12738,21 +12742,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>32.733601</v>
+        <v>37.618999</v>
       </c>
       <c r="H328" t="n">
-        <v>-117.190002</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12762,7 +12766,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12776,21 +12780,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>37.618999</v>
+        <v>37.362598</v>
       </c>
       <c r="H329" t="n">
-        <v>-122.375</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12800,35 +12804,35 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G330" t="n">
-        <v>37.362598</v>
+        <v>52.170799</v>
       </c>
       <c r="H330" t="n">
-        <v>-121.929001</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12838,35 +12842,35 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G331" t="n">
-        <v>52.170799</v>
+        <v>47.449001</v>
       </c>
       <c r="H331" t="n">
-        <v>-106.699997</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12876,7 +12880,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12890,21 +12894,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>47.449001</v>
+        <v>43.582001</v>
       </c>
       <c r="H332" t="n">
-        <v>-122.308998</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12914,7 +12918,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12928,21 +12932,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>43.582001</v>
+        <v>38.748699</v>
       </c>
       <c r="H333" t="n">
-        <v>-96.74189800000001</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12952,7 +12956,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -12966,21 +12970,21 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>38.748699</v>
+        <v>30.3965</v>
       </c>
       <c r="H334" t="n">
-        <v>-90.370003</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12990,7 +12994,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13004,21 +13008,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>30.3965</v>
+        <v>27.9755</v>
       </c>
       <c r="H335" t="n">
-        <v>-84.35030399999999</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13028,35 +13032,35 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G336" t="n">
-        <v>27.9755</v>
+        <v>43.6772</v>
       </c>
       <c r="H336" t="n">
-        <v>-82.533203</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13066,7 +13070,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13080,21 +13084,21 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>43.6772</v>
+        <v>49.193901</v>
       </c>
       <c r="H337" t="n">
-        <v>-79.6306</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YWG</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Winnipeg, MB, Canada</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13104,7 +13108,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Winnipeg</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -13118,21 +13122,21 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>49.193901</v>
+        <v>49.91</v>
       </c>
       <c r="H338" t="n">
-        <v>-123.183998</v>
+        <v>-97.23989899999999</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>CVG</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Cincinnati, United States</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13142,61 +13146,23 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Hebron</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G339" t="n">
-        <v>49.91</v>
+        <v>39.048801</v>
       </c>
       <c r="H339" t="n">
-        <v>-97.23989899999999</v>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" s="1" t="inlineStr">
-        <is>
-          <t>CVG</t>
-        </is>
-      </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>Cincinnati, United States</t>
-        </is>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>Hebron</t>
-        </is>
-      </c>
-      <c r="E340" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="F340" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G340" t="n">
-        <v>39.048801</v>
-      </c>
-      <c r="H340" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by cc096a5e34ba2d3de6e0f9811c5c1c7518a77cf1
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H339"/>
+  <dimension ref="A1:H340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10927,50 +10927,50 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>UDR</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Udaipur, India</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Udaipur</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G281" t="n">
-        <v>35.040199</v>
+        <v>24.617701</v>
       </c>
       <c r="H281" t="n">
-        <v>-106.609001</v>
+        <v>73.896103</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10980,7 +10980,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -10994,21 +10994,21 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H282" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11018,7 +11018,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11032,21 +11032,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H283" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11070,21 +11070,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H284" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11094,7 +11094,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11108,21 +11108,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H285" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11132,7 +11132,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11146,21 +11146,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H286" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11170,7 +11170,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11184,21 +11184,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H287" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11208,7 +11208,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11222,21 +11222,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H288" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11246,35 +11246,35 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G289" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H289" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11284,35 +11284,35 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G290" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H290" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11336,21 +11336,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H291" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11360,7 +11360,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11374,21 +11374,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H292" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11412,21 +11412,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H293" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11436,7 +11436,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11450,21 +11450,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H294" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11474,7 +11474,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11488,21 +11488,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H295" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11512,7 +11512,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11526,21 +11526,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H296" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11564,21 +11564,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H297" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11588,35 +11588,35 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H298" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11626,35 +11626,35 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G299" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H299" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11664,35 +11664,35 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G300" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H300" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11702,7 +11702,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11716,21 +11716,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H301" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11740,7 +11740,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11754,21 +11754,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H302" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11778,7 +11778,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11792,21 +11792,21 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H303" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11816,7 +11816,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11830,21 +11830,21 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H304" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11854,35 +11854,35 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H305" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11892,35 +11892,35 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G306" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H306" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11930,7 +11930,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11944,21 +11944,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H307" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11968,7 +11968,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -11982,21 +11982,21 @@
         </is>
       </c>
       <c r="G308" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H308" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12006,35 +12006,35 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H309" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12044,35 +12044,35 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H310" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12082,7 +12082,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12096,21 +12096,21 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H311" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12120,35 +12120,35 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G312" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H312" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12158,35 +12158,35 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G313" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H313" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12196,7 +12196,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12210,21 +12210,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H314" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12248,21 +12248,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H315" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12286,21 +12286,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H316" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12310,7 +12310,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12324,21 +12324,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H317" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12362,21 +12362,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>39.871899</v>
+        <v>41.3032</v>
       </c>
       <c r="H318" t="n">
-        <v>-75.241096</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12386,7 +12386,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12400,21 +12400,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H319" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12424,7 +12424,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12438,21 +12438,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H320" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12462,7 +12462,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12476,21 +12476,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H321" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12500,35 +12500,35 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G322" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H322" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12538,35 +12538,35 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G323" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H323" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12576,7 +12576,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12590,21 +12590,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H324" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12628,21 +12628,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H325" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12652,7 +12652,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12666,21 +12666,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H326" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12690,7 +12690,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12704,21 +12704,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H327" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12728,7 +12728,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12742,21 +12742,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H328" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12766,7 +12766,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12780,21 +12780,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H329" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12804,35 +12804,35 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G330" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H330" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12842,35 +12842,35 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G331" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H331" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12880,7 +12880,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12894,21 +12894,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H332" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12918,7 +12918,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12932,21 +12932,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H333" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -12970,21 +12970,21 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H334" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12994,7 +12994,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13008,21 +13008,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H335" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13032,35 +13032,35 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G336" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H336" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13070,7 +13070,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13084,21 +13084,21 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H337" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13108,7 +13108,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -13122,47 +13122,85 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>49.91</v>
+        <v>49.193901</v>
       </c>
       <c r="H338" t="n">
-        <v>-97.23989899999999</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G339" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H339" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
+      <c r="B340" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C339" t="inlineStr">
+      <c r="C340" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr">
+      <c r="D340" t="inlineStr">
         <is>
           <t>Hebron</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr">
+      <c r="E340" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F339" t="inlineStr">
+      <c r="F340" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G339" t="n">
+      <c r="G340" t="n">
         <v>39.048801</v>
       </c>
-      <c r="H339" t="n">
+      <c r="H340" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 1917c9e2b2a1f0bb06b68002b07d3a6404471340
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H340"/>
+  <dimension ref="A1:H341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10965,50 +10965,46 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>AIP</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Jalandhar, India</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t>Albuquerque</t>
-        </is>
-      </c>
+          <t>Asia Pacific</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr"/>
       <c r="E282" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G282" t="n">
-        <v>35.040199</v>
+        <v>31.4338</v>
       </c>
       <c r="H282" t="n">
-        <v>-106.609001</v>
+        <v>75.758797</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -11018,7 +11014,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11032,21 +11028,21 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H283" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11056,7 +11052,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11070,21 +11066,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H284" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11094,7 +11090,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11108,21 +11104,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H285" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11132,7 +11128,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11146,21 +11142,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H286" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11170,7 +11166,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11184,21 +11180,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H287" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11208,7 +11204,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11222,21 +11218,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H288" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11246,7 +11242,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11260,21 +11256,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H289" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11284,35 +11280,35 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G290" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H290" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11322,35 +11318,35 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G291" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H291" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11360,7 +11356,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11374,21 +11370,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H292" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11398,7 +11394,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11412,21 +11408,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H293" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11436,7 +11432,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11450,21 +11446,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H294" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11474,7 +11470,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11488,21 +11484,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H295" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11512,7 +11508,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11526,21 +11522,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H296" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11550,7 +11546,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11564,21 +11560,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H297" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11588,7 +11584,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -11602,21 +11598,21 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H298" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11626,35 +11622,35 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G299" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H299" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11664,35 +11660,35 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G300" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H300" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11702,35 +11698,35 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G301" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H301" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11740,7 +11736,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11754,21 +11750,21 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H302" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11778,7 +11774,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11792,21 +11788,21 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H303" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11816,7 +11812,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11830,21 +11826,21 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H304" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11854,7 +11850,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11868,21 +11864,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H305" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11892,35 +11888,35 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G306" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H306" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11930,35 +11926,35 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H307" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11968,7 +11964,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -11982,21 +11978,21 @@
         </is>
       </c>
       <c r="G308" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H308" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12006,7 +12002,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12020,21 +12016,21 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H309" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12044,35 +12040,35 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H310" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12082,35 +12078,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H311" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12120,7 +12116,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12134,21 +12130,21 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H312" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12158,35 +12154,35 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G313" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H313" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12196,35 +12192,35 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G314" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H314" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12234,7 +12230,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12248,21 +12244,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H315" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12272,7 +12268,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12286,21 +12282,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H316" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12310,7 +12306,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12324,21 +12320,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H317" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12348,7 +12344,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12362,21 +12358,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H318" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12386,7 +12382,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12400,21 +12396,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>39.871899</v>
+        <v>41.3032</v>
       </c>
       <c r="H319" t="n">
-        <v>-75.241096</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12424,7 +12420,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12438,21 +12434,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H320" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12462,7 +12458,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12476,21 +12472,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H321" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12500,7 +12496,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12514,21 +12510,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H322" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12538,35 +12534,35 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G323" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H323" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12576,35 +12572,35 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G324" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H324" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12614,7 +12610,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12628,21 +12624,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H325" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12652,7 +12648,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12666,21 +12662,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H326" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12690,7 +12686,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12704,21 +12700,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H327" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12728,7 +12724,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12742,21 +12738,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H328" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12766,7 +12762,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12780,21 +12776,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H329" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12804,7 +12800,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12818,21 +12814,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H330" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12842,35 +12838,35 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G331" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H331" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12880,35 +12876,35 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G332" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H332" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12918,7 +12914,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12932,21 +12928,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H333" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12956,7 +12952,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -12970,21 +12966,21 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H334" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12994,7 +12990,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13008,21 +13004,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H335" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13032,7 +13028,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13046,21 +13042,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H336" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13070,35 +13066,35 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G337" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H337" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13108,7 +13104,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -13122,21 +13118,21 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H338" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13146,7 +13142,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -13160,47 +13156,85 @@
         </is>
       </c>
       <c r="G339" t="n">
-        <v>49.91</v>
+        <v>49.193901</v>
       </c>
       <c r="H339" t="n">
-        <v>-97.23989899999999</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G340" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H340" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B340" t="inlineStr">
+      <c r="B341" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C340" t="inlineStr">
+      <c r="C341" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D340" t="inlineStr">
+      <c r="D341" t="inlineStr">
         <is>
           <t>Hebron</t>
         </is>
       </c>
-      <c r="E340" t="inlineStr">
+      <c r="E341" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F340" t="inlineStr">
+      <c r="F341" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G340" t="n">
+      <c r="G341" t="n">
         <v>39.048801</v>
       </c>
-      <c r="H340" t="n">
+      <c r="H341" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 3894fac4984746b2513daff0320247240f9c5a26
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H341"/>
+  <dimension ref="A1:H342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10999,50 +10999,46 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>LHW</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Lanzhou, China</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Lanzhou</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="G283" t="n">
-        <v>35.040199</v>
-      </c>
-      <c r="H283" t="n">
-        <v>-106.609001</v>
-      </c>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr"/>
+      <c r="H283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -11052,7 +11048,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11066,21 +11062,21 @@
         </is>
       </c>
       <c r="G284" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H284" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11090,7 +11086,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11104,21 +11100,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H285" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11128,7 +11124,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11142,21 +11138,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H286" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11166,7 +11162,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11180,21 +11176,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H287" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11204,7 +11200,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11218,21 +11214,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H288" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11242,7 +11238,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11256,21 +11252,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H289" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11280,7 +11276,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11294,21 +11290,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H290" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11318,35 +11314,35 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G291" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H291" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11356,35 +11352,35 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G292" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H292" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11394,7 +11390,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11408,21 +11404,21 @@
         </is>
       </c>
       <c r="G293" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H293" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11432,7 +11428,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11446,21 +11442,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H294" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11470,7 +11466,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11484,21 +11480,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H295" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11508,7 +11504,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11522,21 +11518,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H296" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11546,7 +11542,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11560,21 +11556,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H297" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11584,7 +11580,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -11598,21 +11594,21 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H298" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11622,7 +11618,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11636,21 +11632,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H299" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11660,35 +11656,35 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G300" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H300" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11698,35 +11694,35 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G301" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H301" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11736,35 +11732,35 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G302" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H302" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11774,7 +11770,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11788,21 +11784,21 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H303" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11812,7 +11808,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11826,21 +11822,21 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H304" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11850,7 +11846,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11864,21 +11860,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H305" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11888,7 +11884,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11902,21 +11898,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H306" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11926,35 +11922,35 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G307" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H307" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11964,35 +11960,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H308" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -12002,7 +11998,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12016,21 +12012,21 @@
         </is>
       </c>
       <c r="G309" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H309" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12040,7 +12036,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12054,21 +12050,21 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H310" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12078,35 +12074,35 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G311" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H311" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12116,35 +12112,35 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G312" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H312" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12154,7 +12150,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12168,21 +12164,21 @@
         </is>
       </c>
       <c r="G313" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H313" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12192,35 +12188,35 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G314" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H314" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12230,35 +12226,35 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G315" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H315" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12268,7 +12264,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12282,21 +12278,21 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H316" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12306,7 +12302,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12320,21 +12316,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H317" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12344,7 +12340,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12358,21 +12354,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H318" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12382,7 +12378,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12396,21 +12392,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H319" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12420,7 +12416,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12434,21 +12430,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>39.871899</v>
+        <v>41.3032</v>
       </c>
       <c r="H320" t="n">
-        <v>-75.241096</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12458,7 +12454,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12472,21 +12468,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H321" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12496,7 +12492,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12510,21 +12506,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H322" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12534,7 +12530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12548,21 +12544,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H323" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12572,35 +12568,35 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G324" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H324" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12610,35 +12606,35 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G325" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H325" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12648,7 +12644,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12662,21 +12658,21 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H326" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12686,7 +12682,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12700,21 +12696,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H327" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12724,7 +12720,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12738,21 +12734,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H328" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12762,7 +12758,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12776,21 +12772,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H329" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12800,7 +12796,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12814,21 +12810,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H330" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12838,7 +12834,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12852,21 +12848,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H331" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12876,35 +12872,35 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G332" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H332" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12914,35 +12910,35 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G333" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H333" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12952,7 +12948,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -12966,21 +12962,21 @@
         </is>
       </c>
       <c r="G334" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H334" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12990,7 +12986,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13004,21 +13000,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H335" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13028,7 +13024,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13042,21 +13038,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H336" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13066,7 +13062,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13080,21 +13076,21 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H337" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13104,35 +13100,35 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G338" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H338" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13142,7 +13138,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -13156,21 +13152,21 @@
         </is>
       </c>
       <c r="G339" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H339" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -13180,7 +13176,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -13194,47 +13190,85 @@
         </is>
       </c>
       <c r="G340" t="n">
-        <v>49.91</v>
+        <v>49.193901</v>
       </c>
       <c r="H340" t="n">
-        <v>-97.23989899999999</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G341" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H341" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B341" t="inlineStr">
+      <c r="B342" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C341" t="inlineStr">
+      <c r="C342" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D341" t="inlineStr">
+      <c r="D342" t="inlineStr">
         <is>
           <t>Hebron</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr">
+      <c r="E342" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F341" t="inlineStr">
+      <c r="F342" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G341" t="n">
+      <c r="G342" t="n">
         <v>39.048801</v>
       </c>
-      <c r="H341" t="n">
+      <c r="H342" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by cc49ca2cc0bde1d3676955665d1e8965dbdb3c4f
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H342"/>
+  <dimension ref="A1:H343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11033,50 +11033,50 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>DYU</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Dushanbe, Tajikistan</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>North America</t>
+          <t>Asia Pacific</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Dushanbe</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Tajikistan</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="G284" t="n">
-        <v>35.040199</v>
+        <v>38.543301</v>
       </c>
       <c r="H284" t="n">
-        <v>-106.609001</v>
+        <v>68.824997</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -11086,7 +11086,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11100,21 +11100,21 @@
         </is>
       </c>
       <c r="G285" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H285" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11124,7 +11124,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11138,21 +11138,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H286" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11162,7 +11162,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11176,21 +11176,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H287" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11200,7 +11200,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11214,21 +11214,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H288" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11238,7 +11238,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11252,21 +11252,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H289" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11276,7 +11276,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11290,21 +11290,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H290" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11314,7 +11314,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11328,21 +11328,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H291" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11352,35 +11352,35 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G292" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H292" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11390,35 +11390,35 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G293" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H293" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11428,7 +11428,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11442,21 +11442,21 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H294" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11466,7 +11466,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11480,21 +11480,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H295" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11518,21 +11518,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H296" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11542,7 +11542,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11556,21 +11556,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H297" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11580,7 +11580,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -11594,21 +11594,21 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H298" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11632,21 +11632,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H299" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11656,7 +11656,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11670,21 +11670,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H300" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11694,35 +11694,35 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G301" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H301" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11732,35 +11732,35 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G302" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H302" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11770,35 +11770,35 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H303" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11808,7 +11808,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11822,21 +11822,21 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H304" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11860,21 +11860,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H305" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11884,7 +11884,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11898,21 +11898,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H306" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11922,7 +11922,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11936,21 +11936,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H307" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11960,35 +11960,35 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G308" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H308" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -11998,35 +11998,35 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H309" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12036,7 +12036,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12050,21 +12050,21 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H310" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12074,7 +12074,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12088,21 +12088,21 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H311" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12112,35 +12112,35 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G312" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H312" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12150,35 +12150,35 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G313" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H313" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12188,7 +12188,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12202,21 +12202,21 @@
         </is>
       </c>
       <c r="G314" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H314" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12226,35 +12226,35 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G315" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H315" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12264,35 +12264,35 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G316" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H316" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12302,7 +12302,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12316,21 +12316,21 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H317" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12340,7 +12340,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12354,21 +12354,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H318" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12378,7 +12378,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12392,21 +12392,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H319" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12416,7 +12416,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12430,21 +12430,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H320" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12454,7 +12454,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12468,21 +12468,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>39.871899</v>
+        <v>41.3032</v>
       </c>
       <c r="H321" t="n">
-        <v>-75.241096</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12492,7 +12492,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12506,21 +12506,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H322" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12530,7 +12530,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12544,21 +12544,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H323" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12568,7 +12568,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12582,21 +12582,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H324" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12606,35 +12606,35 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G325" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H325" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12644,35 +12644,35 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G326" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H326" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12682,7 +12682,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12696,21 +12696,21 @@
         </is>
       </c>
       <c r="G327" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H327" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12720,7 +12720,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12734,21 +12734,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H328" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12758,7 +12758,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12772,21 +12772,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H329" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12810,21 +12810,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H330" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12834,7 +12834,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12848,21 +12848,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H331" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12872,7 +12872,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12886,21 +12886,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H332" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12910,35 +12910,35 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G333" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H333" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12948,35 +12948,35 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G334" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H334" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12986,7 +12986,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13000,21 +13000,21 @@
         </is>
       </c>
       <c r="G335" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H335" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13024,7 +13024,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13038,21 +13038,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H336" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13076,21 +13076,21 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H337" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13100,7 +13100,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -13114,21 +13114,21 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H338" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13138,35 +13138,35 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G339" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H339" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -13176,7 +13176,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -13190,21 +13190,21 @@
         </is>
       </c>
       <c r="G340" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H340" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -13214,7 +13214,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -13228,47 +13228,85 @@
         </is>
       </c>
       <c r="G341" t="n">
-        <v>49.91</v>
+        <v>49.193901</v>
       </c>
       <c r="H341" t="n">
-        <v>-97.23989899999999</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G342" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H342" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B343" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C343" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr">
+      <c r="D343" t="inlineStr">
         <is>
           <t>Hebron</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr">
+      <c r="E343" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F342" t="inlineStr">
+      <c r="F343" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G342" t="n">
+      <c r="G343" t="n">
         <v>39.048801</v>
       </c>
-      <c r="H342" t="n">
+      <c r="H343" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update generated data Triggered by 10ca317792da943f5452a70bebff82bee0967941
</commit_message>
<xml_diff>
--- a/DC-Colos.xlsx
+++ b/DC-Colos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H343"/>
+  <dimension ref="A1:H344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11071,50 +11071,46 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>ABQ</t>
+          <t>LUH</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Albuquerque, NM, United States</t>
+          <t>Ludhiana, India</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>North America</t>
-        </is>
-      </c>
-      <c r="D285" t="inlineStr">
-        <is>
-          <t>Albuquerque</t>
-        </is>
-      </c>
+          <t>Asia Pacific</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr"/>
       <c r="E285" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>India</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="G285" t="n">
-        <v>35.040199</v>
+        <v>30.8547</v>
       </c>
       <c r="H285" t="n">
-        <v>-106.609001</v>
+        <v>75.95259900000001</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>ANC</t>
+          <t>ABQ</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Anchorage, AK, United States</t>
+          <t>Albuquerque, NM, United States</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -11124,7 +11120,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Anchorage</t>
+          <t>Albuquerque</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11138,21 +11134,21 @@
         </is>
       </c>
       <c r="G286" t="n">
-        <v>61.1744</v>
+        <v>35.040199</v>
       </c>
       <c r="H286" t="n">
-        <v>-149.996002</v>
+        <v>-106.609001</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>IAD</t>
+          <t>ANC</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Ashburn, VA, United States</t>
+          <t>Anchorage, AK, United States</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -11162,7 +11158,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Dulles</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11176,21 +11172,21 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>38.9445</v>
+        <v>61.1744</v>
       </c>
       <c r="H287" t="n">
-        <v>-77.455803</v>
+        <v>-149.996002</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>IAD</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Atlanta, GA, United States</t>
+          <t>Ashburn, VA, United States</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -11200,7 +11196,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Dulles</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11214,21 +11210,21 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>33.6367</v>
+        <v>38.9445</v>
       </c>
       <c r="H288" t="n">
-        <v>-84.428101</v>
+        <v>-77.455803</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Austin, TX, United States</t>
+          <t>Atlanta, GA, United States</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -11238,7 +11234,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11252,21 +11248,21 @@
         </is>
       </c>
       <c r="G289" t="n">
-        <v>30.1945</v>
+        <v>33.6367</v>
       </c>
       <c r="H289" t="n">
-        <v>-97.669899</v>
+        <v>-84.428101</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>BGR</t>
+          <t>AUS</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Bangor, ME, United States</t>
+          <t>Austin, TX, United States</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -11276,7 +11272,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Bangor</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11290,21 +11286,21 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>44.8074</v>
+        <v>30.1945</v>
       </c>
       <c r="H290" t="n">
-        <v>-68.828102</v>
+        <v>-97.669899</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>BGR</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Boston, MA, United States</t>
+          <t>Bangor, ME, United States</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -11314,7 +11310,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Bangor</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11328,21 +11324,21 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>42.3643</v>
+        <v>44.8074</v>
       </c>
       <c r="H291" t="n">
-        <v>-71.00520299999999</v>
+        <v>-68.828102</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Buffalo, NY, United States</t>
+          <t>Boston, MA, United States</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -11352,7 +11348,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11366,21 +11362,21 @@
         </is>
       </c>
       <c r="G292" t="n">
-        <v>42.940498</v>
+        <v>42.3643</v>
       </c>
       <c r="H292" t="n">
-        <v>-78.732201</v>
+        <v>-71.00520299999999</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>YYC</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Calgary, AB, Canada</t>
+          <t>Buffalo, NY, United States</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -11390,35 +11386,35 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Calgary</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G293" t="n">
-        <v>51.113899</v>
+        <v>42.940498</v>
       </c>
       <c r="H293" t="n">
-        <v>-114.019997</v>
+        <v>-78.732201</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>CLT</t>
+          <t>YYC</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Charlotte, NC, United States</t>
+          <t>Calgary, AB, Canada</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -11428,35 +11424,35 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Calgary</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G294" t="n">
-        <v>35.214001</v>
+        <v>51.113899</v>
       </c>
       <c r="H294" t="n">
-        <v>-80.9431</v>
+        <v>-114.019997</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>ORD</t>
+          <t>CLT</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Chicago, IL, United States</t>
+          <t>Charlotte, NC, United States</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -11466,7 +11462,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11480,21 +11476,21 @@
         </is>
       </c>
       <c r="G295" t="n">
-        <v>41.9786</v>
+        <v>35.214001</v>
       </c>
       <c r="H295" t="n">
-        <v>-87.90479999999999</v>
+        <v>-80.9431</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ORD</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Cleveland, OH, United States</t>
+          <t>Chicago, IL, United States</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -11504,7 +11500,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11518,21 +11514,21 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>41.411701</v>
+        <v>41.9786</v>
       </c>
       <c r="H296" t="n">
-        <v>-81.8498</v>
+        <v>-87.90479999999999</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>CMH</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Columbus, OH, United States</t>
+          <t>Cleveland, OH, United States</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -11542,7 +11538,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Columbus</t>
+          <t>Cleveland</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11556,21 +11552,21 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>39.998001</v>
+        <v>41.411701</v>
       </c>
       <c r="H297" t="n">
-        <v>-82.891899</v>
+        <v>-81.8498</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>DFW</t>
+          <t>CMH</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Dallas, TX, United States</t>
+          <t>Columbus, OH, United States</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -11580,7 +11576,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Dallas-Fort Worth</t>
+          <t>Columbus</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -11594,21 +11590,21 @@
         </is>
       </c>
       <c r="G298" t="n">
-        <v>32.896801</v>
+        <v>39.998001</v>
       </c>
       <c r="H298" t="n">
-        <v>-97.03800200000001</v>
+        <v>-82.891899</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>DFW</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Denver, CO, United States</t>
+          <t>Dallas, TX, United States</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -11618,7 +11614,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Dallas-Fort Worth</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11632,21 +11628,21 @@
         </is>
       </c>
       <c r="G299" t="n">
-        <v>39.861698</v>
+        <v>32.896801</v>
       </c>
       <c r="H299" t="n">
-        <v>-104.672997</v>
+        <v>-97.03800200000001</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>DTW</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Detroit, MI, United States</t>
+          <t>Denver, CO, United States</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -11656,7 +11652,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Detroit</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11670,21 +11666,21 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>42.212399</v>
+        <v>39.861698</v>
       </c>
       <c r="H300" t="n">
-        <v>-83.35340100000001</v>
+        <v>-104.672997</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>RDU</t>
+          <t>DTW</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Durham, NC, United States</t>
+          <t>Detroit, MI, United States</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -11694,7 +11690,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Raleigh/Durham</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11708,21 +11704,21 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>35.877602</v>
+        <v>42.212399</v>
       </c>
       <c r="H301" t="n">
-        <v>-78.787498</v>
+        <v>-83.35340100000001</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>GDL</t>
+          <t>RDU</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Guadalajara, Mexico</t>
+          <t>Durham, NC, United States</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -11732,35 +11728,35 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Guadalajara</t>
+          <t>Raleigh/Durham</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G302" t="n">
-        <v>20.521799</v>
+        <v>35.877602</v>
       </c>
       <c r="H302" t="n">
-        <v>-103.310997</v>
+        <v>-78.787498</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>YHZ</t>
+          <t>GDL</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Halifax, Canada</t>
+          <t>Guadalajara, Mexico</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -11770,35 +11766,35 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Halifax</t>
+          <t>Guadalajara</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>44.880798</v>
+        <v>20.521799</v>
       </c>
       <c r="H303" t="n">
-        <v>-63.508598</v>
+        <v>-103.310997</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>HNL</t>
+          <t>YHZ</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Honolulu, HI, United States</t>
+          <t>Halifax, Canada</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -11808,35 +11804,35 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Honolulu</t>
+          <t>Halifax</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G304" t="n">
-        <v>21.318701</v>
+        <v>44.880798</v>
       </c>
       <c r="H304" t="n">
-        <v>-157.921997</v>
+        <v>-63.508598</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>IAH</t>
+          <t>HNL</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Houston, TX, United States</t>
+          <t>Honolulu, HI, United States</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -11846,7 +11842,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Honolulu</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -11860,21 +11856,21 @@
         </is>
       </c>
       <c r="G305" t="n">
-        <v>29.9844</v>
+        <v>21.318701</v>
       </c>
       <c r="H305" t="n">
-        <v>-95.34139999999999</v>
+        <v>-157.921997</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>IAH</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Indianapolis, IN, United States</t>
+          <t>Houston, TX, United States</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -11884,7 +11880,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Indianapolis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -11898,21 +11894,21 @@
         </is>
       </c>
       <c r="G306" t="n">
-        <v>39.7173</v>
+        <v>29.9844</v>
       </c>
       <c r="H306" t="n">
-        <v>-86.294403</v>
+        <v>-95.34139999999999</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>JAX</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, United States</t>
+          <t>Indianapolis, IN, United States</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -11922,7 +11918,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Indianapolis</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -11936,21 +11932,21 @@
         </is>
       </c>
       <c r="G307" t="n">
-        <v>30.494101</v>
+        <v>39.7173</v>
       </c>
       <c r="H307" t="n">
-        <v>-81.68789700000001</v>
+        <v>-86.294403</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>MCI</t>
+          <t>JAX</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Kansas City, MO, United States</t>
+          <t>Jacksonville, FL, United States</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -11960,7 +11956,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -11974,21 +11970,21 @@
         </is>
       </c>
       <c r="G308" t="n">
-        <v>39.2976</v>
+        <v>30.494101</v>
       </c>
       <c r="H308" t="n">
-        <v>-94.713898</v>
+        <v>-81.68789700000001</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>KIN</t>
+          <t>MCI</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Kingston, Jamaica</t>
+          <t>Kansas City, MO, United States</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -11998,35 +11994,35 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Kingston</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Jamaica</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>JM</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G309" t="n">
-        <v>17.935699</v>
+        <v>39.2976</v>
       </c>
       <c r="H309" t="n">
-        <v>-76.787498</v>
+        <v>-94.713898</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>LAS</t>
+          <t>KIN</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Las Vegas, NV, United States</t>
+          <t>Kingston, Jamaica</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -12036,35 +12032,35 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Las Vegas</t>
+          <t>Kingston</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Jamaica</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="G310" t="n">
-        <v>36.080101</v>
+        <v>17.935699</v>
       </c>
       <c r="H310" t="n">
-        <v>-115.152</v>
+        <v>-76.787498</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>LAS</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, United States</t>
+          <t>Las Vegas, NV, United States</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -12074,7 +12070,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Las Vegas</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12088,21 +12084,21 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>33.942501</v>
+        <v>36.080101</v>
       </c>
       <c r="H311" t="n">
-        <v>-118.407997</v>
+        <v>-115.152</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>MEM</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Memphis, TN, United States</t>
+          <t>Los Angeles, CA, United States</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -12112,7 +12108,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12126,21 +12122,21 @@
         </is>
       </c>
       <c r="G312" t="n">
-        <v>35.0424</v>
+        <v>33.942501</v>
       </c>
       <c r="H312" t="n">
-        <v>-89.97669999999999</v>
+        <v>-118.407997</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>MEX</t>
+          <t>MEM</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Mexico City, Mexico</t>
+          <t>Memphis, TN, United States</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -12150,35 +12146,35 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Mexico City</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G313" t="n">
-        <v>19.4363</v>
+        <v>35.0424</v>
       </c>
       <c r="H313" t="n">
-        <v>-99.072098</v>
+        <v>-89.97669999999999</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>MEX</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Miami, FL, United States</t>
+          <t>Mexico City, Mexico</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -12188,35 +12184,35 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Mexico City</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G314" t="n">
-        <v>25.7932</v>
+        <v>19.4363</v>
       </c>
       <c r="H314" t="n">
-        <v>-80.290604</v>
+        <v>-99.072098</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>MSP</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Minneapolis, MN, United States</t>
+          <t>Miami, FL, United States</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -12226,7 +12222,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12240,21 +12236,21 @@
         </is>
       </c>
       <c r="G315" t="n">
-        <v>44.882</v>
+        <v>25.7932</v>
       </c>
       <c r="H315" t="n">
-        <v>-93.221802</v>
+        <v>-80.290604</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="1" t="inlineStr">
         <is>
-          <t>YUL</t>
+          <t>MSP</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Minneapolis, MN, United States</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -12264,35 +12260,35 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Montreal</t>
+          <t>Minneapolis</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G316" t="n">
-        <v>45.4706</v>
+        <v>44.882</v>
       </c>
       <c r="H316" t="n">
-        <v>-73.740799</v>
+        <v>-93.221802</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="1" t="inlineStr">
         <is>
-          <t>BNA</t>
+          <t>YUL</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Nashville, United States</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12302,35 +12298,35 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Montreal</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G317" t="n">
-        <v>36.1245</v>
+        <v>45.4706</v>
       </c>
       <c r="H317" t="n">
-        <v>-86.6782</v>
+        <v>-73.740799</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="1" t="inlineStr">
         <is>
-          <t>EWR</t>
+          <t>BNA</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Newark, NJ, United States</t>
+          <t>Nashville, United States</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -12340,7 +12336,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Newark</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12354,21 +12350,21 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>40.692501</v>
+        <v>36.1245</v>
       </c>
       <c r="H318" t="n">
-        <v>-74.168701</v>
+        <v>-86.6782</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="1" t="inlineStr">
         <is>
-          <t>ORF</t>
+          <t>EWR</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Norfolk, VA, United States</t>
+          <t>Newark, NJ, United States</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12378,7 +12374,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Norfolk</t>
+          <t>Newark</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12392,21 +12388,21 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>36.8946</v>
+        <v>40.692501</v>
       </c>
       <c r="H319" t="n">
-        <v>-76.20120199999999</v>
+        <v>-74.168701</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="1" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>ORF</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Oklahoma City, OK, United States</t>
+          <t>Norfolk, VA, United States</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -12416,7 +12412,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Norfolk</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12430,21 +12426,21 @@
         </is>
       </c>
       <c r="G320" t="n">
-        <v>35.393101</v>
+        <v>36.8946</v>
       </c>
       <c r="H320" t="n">
-        <v>-97.6007</v>
+        <v>-76.20120199999999</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="1" t="inlineStr">
         <is>
-          <t>OMA</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Omaha, NE, United States</t>
+          <t>Oklahoma City, OK, United States</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12454,7 +12450,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Oklahoma City</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12468,21 +12464,21 @@
         </is>
       </c>
       <c r="G321" t="n">
-        <v>41.3032</v>
+        <v>35.393101</v>
       </c>
       <c r="H321" t="n">
-        <v>-95.894096</v>
+        <v>-97.6007</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="1" t="inlineStr">
         <is>
-          <t>PHL</t>
+          <t>OMA</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Philadelphia, United States</t>
+          <t>Omaha, NE, United States</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -12492,7 +12488,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Philadelphia</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12506,21 +12502,21 @@
         </is>
       </c>
       <c r="G322" t="n">
-        <v>39.871899</v>
+        <v>41.3032</v>
       </c>
       <c r="H322" t="n">
-        <v>-75.241096</v>
+        <v>-95.894096</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="1" t="inlineStr">
         <is>
-          <t>PHX</t>
+          <t>PHL</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Phoenix, AZ, United States</t>
+          <t>Philadelphia, United States</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -12530,7 +12526,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Philadelphia</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12544,21 +12540,21 @@
         </is>
       </c>
       <c r="G323" t="n">
-        <v>33.434299</v>
+        <v>39.871899</v>
       </c>
       <c r="H323" t="n">
-        <v>-112.012001</v>
+        <v>-75.241096</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="1" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>PHX</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA, United States</t>
+          <t>Phoenix, AZ, United States</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -12568,7 +12564,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Pittsburgh</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12582,21 +12578,21 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>40.491501</v>
+        <v>33.434299</v>
       </c>
       <c r="H324" t="n">
-        <v>-80.23290299999999</v>
+        <v>-112.012001</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="1" t="inlineStr">
         <is>
-          <t>PDX</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Portland, OR, United States</t>
+          <t>Pittsburgh, PA, United States</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -12606,7 +12602,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Portland</t>
+          <t>Pittsburgh</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12620,21 +12616,21 @@
         </is>
       </c>
       <c r="G325" t="n">
-        <v>45.588699</v>
+        <v>40.491501</v>
       </c>
       <c r="H325" t="n">
-        <v>-122.598</v>
+        <v>-80.23290299999999</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="1" t="inlineStr">
         <is>
-          <t>QRO</t>
+          <t>PDX</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Queretaro, MX, Mexico</t>
+          <t>Portland, OR, United States</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -12644,35 +12640,35 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Queretaro</t>
+          <t>Portland</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G326" t="n">
-        <v>20.6173</v>
+        <v>45.588699</v>
       </c>
       <c r="H326" t="n">
-        <v>-100.185997</v>
+        <v>-122.598</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="1" t="inlineStr">
         <is>
-          <t>RIC</t>
+          <t>QRO</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Richmond, VA, United States</t>
+          <t>Queretaro, MX, Mexico</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -12682,35 +12678,35 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Queretaro</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="G327" t="n">
-        <v>37.505199</v>
+        <v>20.6173</v>
       </c>
       <c r="H327" t="n">
-        <v>-77.31970200000001</v>
+        <v>-100.185997</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="1" t="inlineStr">
         <is>
-          <t>SMF</t>
+          <t>RIC</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Sacramento, CA, United States</t>
+          <t>Richmond, VA, United States</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -12720,7 +12716,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Sacramento</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12734,21 +12730,21 @@
         </is>
       </c>
       <c r="G328" t="n">
-        <v>38.6954</v>
+        <v>37.505199</v>
       </c>
       <c r="H328" t="n">
-        <v>-121.591003</v>
+        <v>-77.31970200000001</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="1" t="inlineStr">
         <is>
-          <t>SLC</t>
+          <t>SMF</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, United States</t>
+          <t>Sacramento, CA, United States</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -12758,7 +12754,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Salt Lake City</t>
+          <t>Sacramento</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12772,21 +12768,21 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>40.788399</v>
+        <v>38.6954</v>
       </c>
       <c r="H329" t="n">
-        <v>-111.977997</v>
+        <v>-121.591003</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="1" t="inlineStr">
         <is>
-          <t>SAT</t>
+          <t>SLC</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>San Antonio, TX, United States</t>
+          <t>Salt Lake City, UT, United States</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -12796,7 +12792,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Salt Lake City</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12810,21 +12806,21 @@
         </is>
       </c>
       <c r="G330" t="n">
-        <v>29.533701</v>
+        <v>40.788399</v>
       </c>
       <c r="H330" t="n">
-        <v>-98.469803</v>
+        <v>-111.977997</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="1" t="inlineStr">
         <is>
-          <t>SAN</t>
+          <t>SAT</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>San Diego, CA, United States</t>
+          <t>San Antonio, TX, United States</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -12834,7 +12830,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>San Diego</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -12848,21 +12844,21 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>32.733601</v>
+        <v>29.533701</v>
       </c>
       <c r="H331" t="n">
-        <v>-117.190002</v>
+        <v>-98.469803</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="1" t="inlineStr">
         <is>
-          <t>SFO</t>
+          <t>SAN</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>San Diego, CA, United States</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -12872,7 +12868,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>San Diego</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -12886,21 +12882,21 @@
         </is>
       </c>
       <c r="G332" t="n">
-        <v>37.618999</v>
+        <v>32.733601</v>
       </c>
       <c r="H332" t="n">
-        <v>-122.375</v>
+        <v>-117.190002</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="1" t="inlineStr">
         <is>
-          <t>SJC</t>
+          <t>SFO</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>San Jose, CA, United States</t>
+          <t>San Francisco, CA, United States</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -12910,7 +12906,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>San Jose</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -12924,21 +12920,21 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>37.362598</v>
+        <v>37.618999</v>
       </c>
       <c r="H333" t="n">
-        <v>-121.929001</v>
+        <v>-122.375</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="1" t="inlineStr">
         <is>
-          <t>YXE</t>
+          <t>SJC</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Saskatoon, SK, Canada</t>
+          <t>San Jose, CA, United States</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -12948,35 +12944,35 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Saskatoon</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G334" t="n">
-        <v>52.170799</v>
+        <v>37.362598</v>
       </c>
       <c r="H334" t="n">
-        <v>-106.699997</v>
+        <v>-121.929001</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="1" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>YXE</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Seattle, WA, United States</t>
+          <t>Saskatoon, SK, Canada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -12986,35 +12982,35 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Seattle</t>
+          <t>Saskatoon</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="G335" t="n">
-        <v>47.449001</v>
+        <v>52.170799</v>
       </c>
       <c r="H335" t="n">
-        <v>-122.308998</v>
+        <v>-106.699997</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="1" t="inlineStr">
         <is>
-          <t>FSD</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Sioux Falls, SD, United States</t>
+          <t>Seattle, WA, United States</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -13024,7 +13020,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Seattle</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13038,21 +13034,21 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>43.582001</v>
+        <v>47.449001</v>
       </c>
       <c r="H336" t="n">
-        <v>-96.74189800000001</v>
+        <v>-122.308998</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="1" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>FSD</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>St. Louis, MO, United States</t>
+          <t>Sioux Falls, SD, United States</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -13062,7 +13058,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13076,21 +13072,21 @@
         </is>
       </c>
       <c r="G337" t="n">
-        <v>38.748699</v>
+        <v>43.582001</v>
       </c>
       <c r="H337" t="n">
-        <v>-90.370003</v>
+        <v>-96.74189800000001</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="1" t="inlineStr">
         <is>
-          <t>TLH</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Tallahassee, FL, United States</t>
+          <t>St. Louis, MO, United States</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -13100,7 +13096,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Tallahassee</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -13114,21 +13110,21 @@
         </is>
       </c>
       <c r="G338" t="n">
-        <v>30.3965</v>
+        <v>38.748699</v>
       </c>
       <c r="H338" t="n">
-        <v>-84.35030399999999</v>
+        <v>-90.370003</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="1" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>TLH</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Tampa, FL, United States</t>
+          <t>Tallahassee, FL, United States</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -13138,7 +13134,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Tallahassee</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -13152,21 +13148,21 @@
         </is>
       </c>
       <c r="G339" t="n">
-        <v>27.9755</v>
+        <v>30.3965</v>
       </c>
       <c r="H339" t="n">
-        <v>-82.533203</v>
+        <v>-84.35030399999999</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="1" t="inlineStr">
         <is>
-          <t>YYZ</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Toronto, ON, Canada</t>
+          <t>Tampa, FL, United States</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -13176,35 +13172,35 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Toronto</t>
+          <t>Tampa</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G340" t="n">
-        <v>43.6772</v>
+        <v>27.9755</v>
       </c>
       <c r="H340" t="n">
-        <v>-79.6306</v>
+        <v>-82.533203</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="1" t="inlineStr">
         <is>
-          <t>YVR</t>
+          <t>YYZ</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Vancouver, BC, Canada</t>
+          <t>Toronto, ON, Canada</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -13214,7 +13210,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Vancouver</t>
+          <t>Toronto</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -13228,21 +13224,21 @@
         </is>
       </c>
       <c r="G341" t="n">
-        <v>49.193901</v>
+        <v>43.6772</v>
       </c>
       <c r="H341" t="n">
-        <v>-123.183998</v>
+        <v>-79.6306</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="1" t="inlineStr">
         <is>
-          <t>YWG</t>
+          <t>YVR</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Winnipeg, MB, Canada</t>
+          <t>Vancouver, BC, Canada</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -13252,7 +13248,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Winnipeg</t>
+          <t>Vancouver</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -13266,47 +13262,85 @@
         </is>
       </c>
       <c r="G342" t="n">
-        <v>49.91</v>
+        <v>49.193901</v>
       </c>
       <c r="H342" t="n">
-        <v>-97.23989899999999</v>
+        <v>-123.183998</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="1" t="inlineStr">
         <is>
+          <t>YWG</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Winnipeg, MB, Canada</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G343" t="n">
+        <v>49.91</v>
+      </c>
+      <c r="H343" t="n">
+        <v>-97.23989899999999</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="1" t="inlineStr">
+        <is>
           <t>CVG</t>
         </is>
       </c>
-      <c r="B343" t="inlineStr">
+      <c r="B344" t="inlineStr">
         <is>
           <t>Cincinnati, United States</t>
         </is>
       </c>
-      <c r="C343" t="inlineStr">
+      <c r="C344" t="inlineStr">
         <is>
           <t>North America</t>
         </is>
       </c>
-      <c r="D343" t="inlineStr">
+      <c r="D344" t="inlineStr">
         <is>
           <t>Hebron</t>
         </is>
       </c>
-      <c r="E343" t="inlineStr">
+      <c r="E344" t="inlineStr">
         <is>
           <t>United States</t>
         </is>
       </c>
-      <c r="F343" t="inlineStr">
+      <c r="F344" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G343" t="n">
+      <c r="G344" t="n">
         <v>39.048801</v>
       </c>
-      <c r="H343" t="n">
+      <c r="H344" t="n">
         <v>-84.667801</v>
       </c>
     </row>

</xml_diff>